<commit_message>
reporting functions with excel support
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/python/epsilonPhi/core/reporting/formatted_excel.xlsx
+++ b/epsilon-phi-core/src/python/epsilonPhi/core/reporting/formatted_excel.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/python/epsilonPhi/core/reporting/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/python/epsilonPhi/core/reporting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA74BDD-380D-4847-B951-17347511899F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86582B5F-B302-1F41-8EA7-2F5FF1A2D7BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="5020" windowWidth="35520" windowHeight="23160" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3100" yWindow="500" windowWidth="33600" windowHeight="19040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
     <sheet name="Portfolios" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="Risk-Metrics" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="Factor Charts" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="Assumptions" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Assumptions" sheetId="5" r:id="rId5"/>
     <sheet name="RAW WEIGHTS" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet5" sheetId="11" r:id="rId7"/>
     <sheet name="Sheet3" sheetId="9" r:id="rId8"/>
@@ -4008,7 +4008,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="mmm\ yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="mmm\ yyyy;@"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -4030,6 +4030,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -4641,45 +4642,6 @@
     <xf numFmtId="164" fontId="6" fillId="3" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4691,9 +4653,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4711,7 +4670,7 @@
     <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -4721,7 +4680,7 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4730,7 +4689,7 @@
     <xf numFmtId="2" fontId="0" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4743,7 +4702,7 @@
     <xf numFmtId="2" fontId="0" fillId="14" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4784,6 +4743,48 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6735,232 +6736,232 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="57"/>
-      <c r="B1" s="103" t="s">
+      <c r="B1" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="103"/>
-      <c r="D1" s="103" t="s">
+      <c r="C1" s="133"/>
+      <c r="D1" s="133" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="103"/>
-      <c r="F1" s="103" t="s">
+      <c r="E1" s="133"/>
+      <c r="F1" s="133" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="103"/>
-      <c r="H1" s="103" t="s">
+      <c r="G1" s="133"/>
+      <c r="H1" s="133" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="104"/>
+      <c r="I1" s="139"/>
     </row>
     <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="105">
+      <c r="B2" s="132">
         <v>0.745</v>
       </c>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105" t="s">
+      <c r="C2" s="132"/>
+      <c r="D2" s="132" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105">
+      <c r="E2" s="132"/>
+      <c r="F2" s="132">
         <v>0.36</v>
       </c>
-      <c r="G2" s="105"/>
-      <c r="H2" s="105">
+      <c r="G2" s="132"/>
+      <c r="H2" s="132">
         <v>0.15</v>
       </c>
-      <c r="I2" s="105"/>
+      <c r="I2" s="132"/>
     </row>
     <row r="3" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="98">
+      <c r="B3" s="134">
         <v>0.02</v>
       </c>
-      <c r="C3" s="98"/>
-      <c r="D3" s="98">
+      <c r="C3" s="134"/>
+      <c r="D3" s="134">
         <v>0.03</v>
       </c>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98">
+      <c r="E3" s="134"/>
+      <c r="F3" s="134">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G3" s="98"/>
-      <c r="H3" s="98">
+      <c r="G3" s="134"/>
+      <c r="H3" s="134">
         <v>5.5E-2</v>
       </c>
-      <c r="I3" s="98"/>
+      <c r="I3" s="134"/>
     </row>
     <row r="4" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="98">
+      <c r="B4" s="134">
         <v>0.14000000000000001</v>
       </c>
-      <c r="C4" s="98"/>
-      <c r="D4" s="98">
+      <c r="C4" s="134"/>
+      <c r="D4" s="134">
         <v>0.22500000000000001</v>
       </c>
-      <c r="E4" s="98"/>
-      <c r="F4" s="98">
+      <c r="E4" s="134"/>
+      <c r="F4" s="134">
         <v>0.35499999999999998</v>
       </c>
-      <c r="G4" s="98"/>
-      <c r="H4" s="98">
+      <c r="G4" s="134"/>
+      <c r="H4" s="134">
         <v>0.505</v>
       </c>
-      <c r="I4" s="98"/>
+      <c r="I4" s="134"/>
     </row>
     <row r="5" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="98">
+      <c r="B5" s="134">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C5" s="98"/>
-      <c r="D5" s="98">
+      <c r="C5" s="134"/>
+      <c r="D5" s="134">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E5" s="98"/>
-      <c r="F5" s="98">
+      <c r="E5" s="134"/>
+      <c r="F5" s="134">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G5" s="98"/>
-      <c r="H5" s="98">
+      <c r="G5" s="134"/>
+      <c r="H5" s="134">
         <v>0.03</v>
       </c>
-      <c r="I5" s="98"/>
+      <c r="I5" s="134"/>
     </row>
     <row r="6" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="98">
+      <c r="B6" s="134">
         <v>0.04</v>
       </c>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98">
+      <c r="C6" s="134"/>
+      <c r="D6" s="134">
         <v>5.5E-2</v>
       </c>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98">
+      <c r="E6" s="134"/>
+      <c r="F6" s="134">
         <v>0.12</v>
       </c>
-      <c r="G6" s="98"/>
-      <c r="H6" s="98">
+      <c r="G6" s="134"/>
+      <c r="H6" s="134">
         <v>0.185</v>
       </c>
-      <c r="I6" s="98"/>
+      <c r="I6" s="134"/>
     </row>
     <row r="7" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="61" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="99">
+      <c r="B7" s="138">
         <v>0.04</v>
       </c>
-      <c r="C7" s="99"/>
-      <c r="D7" s="99">
+      <c r="C7" s="138"/>
+      <c r="D7" s="138">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E7" s="99"/>
-      <c r="F7" s="99">
+      <c r="E7" s="138"/>
+      <c r="F7" s="138">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G7" s="99"/>
-      <c r="H7" s="99">
+      <c r="G7" s="138"/>
+      <c r="H7" s="138">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I7" s="99"/>
+      <c r="I7" s="138"/>
     </row>
     <row r="8" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="100">
+      <c r="B8" s="137">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="C8" s="100"/>
-      <c r="D8" s="100">
+      <c r="C8" s="137"/>
+      <c r="D8" s="137">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E8" s="100"/>
-      <c r="F8" s="100">
+      <c r="E8" s="137"/>
+      <c r="F8" s="137">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G8" s="100"/>
-      <c r="H8" s="100">
+      <c r="G8" s="137"/>
+      <c r="H8" s="137">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="I8" s="100"/>
+      <c r="I8" s="137"/>
     </row>
     <row r="9" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="101">
+      <c r="B9" s="136">
         <v>0.6</v>
       </c>
-      <c r="C9" s="101"/>
-      <c r="D9" s="101">
+      <c r="C9" s="136"/>
+      <c r="D9" s="136">
         <v>0.59</v>
       </c>
-      <c r="E9" s="101"/>
-      <c r="F9" s="101">
+      <c r="E9" s="136"/>
+      <c r="F9" s="136">
         <v>0.53</v>
       </c>
-      <c r="G9" s="101"/>
-      <c r="H9" s="101">
+      <c r="G9" s="136"/>
+      <c r="H9" s="136">
         <v>0.49</v>
       </c>
-      <c r="I9" s="101"/>
+      <c r="I9" s="136"/>
     </row>
     <row r="10" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="62" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="98">
+      <c r="B10" s="134">
         <v>3.1E-2</v>
       </c>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98">
+      <c r="C10" s="134"/>
+      <c r="D10" s="134">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98">
+      <c r="E10" s="134"/>
+      <c r="F10" s="134">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="G10" s="98"/>
-      <c r="H10" s="98">
+      <c r="G10" s="134"/>
+      <c r="H10" s="134">
         <v>0.10299999999999999</v>
       </c>
-      <c r="I10" s="98"/>
+      <c r="I10" s="134"/>
     </row>
     <row r="11" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="62" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="102" t="s">
+      <c r="B11" s="135" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="102"/>
-      <c r="D11" s="102" t="s">
+      <c r="C11" s="135"/>
+      <c r="D11" s="135" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="102"/>
-      <c r="F11" s="102" t="s">
+      <c r="E11" s="135"/>
+      <c r="F11" s="135" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="102"/>
-      <c r="H11" s="102" t="s">
+      <c r="G11" s="135"/>
+      <c r="H11" s="135" t="s">
         <v>36</v>
       </c>
-      <c r="I11" s="102"/>
+      <c r="I11" s="135"/>
     </row>
     <row r="12" spans="1:9" s="10" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="63" t="s">
@@ -7253,64 +7254,64 @@
       <c r="A23" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="96">
+      <c r="B23" s="140">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="C23" s="96"/>
-      <c r="D23" s="96">
+      <c r="C23" s="140"/>
+      <c r="D23" s="140">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="E23" s="96"/>
-      <c r="F23" s="96">
+      <c r="E23" s="140"/>
+      <c r="F23" s="140">
         <v>6.3E-2</v>
       </c>
-      <c r="G23" s="96"/>
-      <c r="H23" s="96">
+      <c r="G23" s="140"/>
+      <c r="H23" s="140">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="I23" s="96"/>
+      <c r="I23" s="140"/>
     </row>
     <row r="24" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="96">
+      <c r="B24" s="140">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C24" s="96"/>
-      <c r="D24" s="96">
+      <c r="C24" s="140"/>
+      <c r="D24" s="140">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="E24" s="96"/>
-      <c r="F24" s="96">
+      <c r="E24" s="140"/>
+      <c r="F24" s="140">
         <v>0.16200000000000001</v>
       </c>
-      <c r="G24" s="96"/>
-      <c r="H24" s="96">
+      <c r="G24" s="140"/>
+      <c r="H24" s="140">
         <v>0.24299999999999999</v>
       </c>
-      <c r="I24" s="96"/>
+      <c r="I24" s="140"/>
     </row>
     <row r="25" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="B25" s="97">
+      <c r="B25" s="141">
         <v>0</v>
       </c>
-      <c r="C25" s="97"/>
-      <c r="D25" s="97">
+      <c r="C25" s="141"/>
+      <c r="D25" s="141">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="E25" s="97"/>
-      <c r="F25" s="97">
+      <c r="E25" s="141"/>
+      <c r="F25" s="141">
         <v>0.14899999999999999</v>
       </c>
-      <c r="G25" s="97"/>
-      <c r="H25" s="97">
+      <c r="G25" s="141"/>
+      <c r="H25" s="141">
         <v>0.253</v>
       </c>
-      <c r="I25" s="97"/>
+      <c r="I25" s="141"/>
     </row>
     <row r="26" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="71" t="s">
@@ -7329,64 +7330,64 @@
       <c r="A27" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="96">
+      <c r="B27" s="140">
         <v>0.23799999999999999</v>
       </c>
-      <c r="C27" s="96"/>
-      <c r="D27" s="96">
+      <c r="C27" s="140"/>
+      <c r="D27" s="140">
         <v>0.27900000000000003</v>
       </c>
-      <c r="E27" s="96"/>
-      <c r="F27" s="96">
+      <c r="E27" s="140"/>
+      <c r="F27" s="140">
         <v>0.314</v>
       </c>
-      <c r="G27" s="96"/>
-      <c r="H27" s="96">
+      <c r="G27" s="140"/>
+      <c r="H27" s="140">
         <v>0.33700000000000002</v>
       </c>
-      <c r="I27" s="96"/>
+      <c r="I27" s="140"/>
     </row>
     <row r="28" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="96">
+      <c r="B28" s="140">
         <v>0.04</v>
       </c>
-      <c r="C28" s="96"/>
-      <c r="D28" s="96">
+      <c r="C28" s="140"/>
+      <c r="D28" s="140">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="E28" s="96"/>
-      <c r="F28" s="96">
+      <c r="E28" s="140"/>
+      <c r="F28" s="140">
         <v>0.14299999999999999</v>
       </c>
-      <c r="G28" s="96"/>
-      <c r="H28" s="96">
+      <c r="G28" s="140"/>
+      <c r="H28" s="140">
         <v>0.187</v>
       </c>
-      <c r="I28" s="96"/>
+      <c r="I28" s="140"/>
     </row>
     <row r="29" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="96">
+      <c r="B29" s="140">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C29" s="96"/>
-      <c r="D29" s="96">
+      <c r="C29" s="140"/>
+      <c r="D29" s="140">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="E29" s="96"/>
-      <c r="F29" s="96">
+      <c r="E29" s="140"/>
+      <c r="F29" s="140">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G29" s="96"/>
-      <c r="H29" s="96">
+      <c r="G29" s="140"/>
+      <c r="H29" s="140">
         <v>0.108</v>
       </c>
-      <c r="I29" s="96"/>
+      <c r="I29" s="140"/>
     </row>
     <row r="30" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="63" t="s">
@@ -7780,11 +7781,56 @@
     </row>
   </sheetData>
   <mergeCells count="68">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D9:E9"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="B5:C5"/>
@@ -7798,56 +7844,11 @@
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B14:I21">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
@@ -8031,16 +8032,16 @@
   <sheetData>
     <row r="1" spans="1:16" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23"/>
-      <c r="B1" s="108" t="s">
+      <c r="B1" s="144" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="E1" s="144"/>
+      <c r="F1" s="144"/>
+      <c r="G1" s="144"/>
+      <c r="H1" s="144"/>
+      <c r="I1" s="144"/>
       <c r="J1" s="25"/>
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
@@ -8048,13 +8049,13 @@
     </row>
     <row r="2" spans="1:16" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="26"/>
-      <c r="B2" s="106" t="s">
+      <c r="B2" s="142" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="106"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
       <c r="G2" s="28" t="s">
         <v>32</v>
       </c>
@@ -9867,7 +9868,7 @@
       <c r="B2" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="C2" s="110" t="s">
+      <c r="C2" s="97" t="s">
         <v>163</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -9879,7 +9880,7 @@
       <c r="F2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="110" t="s">
+      <c r="G2" s="97" t="s">
         <v>165</v>
       </c>
       <c r="H2" s="3" t="s">
@@ -9922,10 +9923,10 @@
       <c r="H4" s="3">
         <v>1</v>
       </c>
-      <c r="I4" s="109">
+      <c r="I4" s="96">
         <v>34365</v>
       </c>
-      <c r="J4" s="109">
+      <c r="J4" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -9954,10 +9955,10 @@
       <c r="H5" s="3">
         <v>1</v>
       </c>
-      <c r="I5" s="109">
+      <c r="I5" s="96">
         <v>34365</v>
       </c>
-      <c r="J5" s="109">
+      <c r="J5" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -9986,10 +9987,10 @@
       <c r="H6" s="3">
         <v>1</v>
       </c>
-      <c r="I6" s="109">
+      <c r="I6" s="96">
         <v>34365</v>
       </c>
-      <c r="J6" s="109">
+      <c r="J6" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10023,10 +10024,10 @@
       <c r="H8" s="3">
         <v>0</v>
       </c>
-      <c r="I8" s="109">
+      <c r="I8" s="96">
         <v>26723</v>
       </c>
-      <c r="J8" s="109">
+      <c r="J8" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10055,10 +10056,10 @@
       <c r="H9" s="3">
         <v>0</v>
       </c>
-      <c r="I9" s="109">
+      <c r="I9" s="96">
         <v>33662</v>
       </c>
-      <c r="J9" s="109">
+      <c r="J9" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10092,10 +10093,10 @@
       <c r="H11" s="3">
         <v>0</v>
       </c>
-      <c r="I11" s="109">
+      <c r="I11" s="96">
         <v>30589</v>
       </c>
-      <c r="J11" s="109">
+      <c r="J11" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10129,10 +10130,10 @@
       <c r="H13" s="3">
         <v>0</v>
       </c>
-      <c r="I13" s="109">
+      <c r="I13" s="96">
         <v>30589</v>
       </c>
-      <c r="J13" s="109">
+      <c r="J13" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10161,10 +10162,10 @@
       <c r="H14" s="3">
         <v>0</v>
       </c>
-      <c r="I14" s="109">
+      <c r="I14" s="96">
         <v>30650</v>
       </c>
-      <c r="J14" s="109">
+      <c r="J14" s="96">
         <v>44925</v>
       </c>
     </row>
@@ -10193,10 +10194,10 @@
       <c r="H15" s="3">
         <v>0</v>
       </c>
-      <c r="I15" s="109">
+      <c r="I15" s="96">
         <v>30680</v>
       </c>
-      <c r="J15" s="109">
+      <c r="J15" s="96">
         <v>44925</v>
       </c>
     </row>
@@ -10230,10 +10231,10 @@
       <c r="H17" s="3">
         <v>0</v>
       </c>
-      <c r="I17" s="109">
+      <c r="I17" s="96">
         <v>25598</v>
       </c>
-      <c r="J17" s="109">
+      <c r="J17" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10262,10 +10263,10 @@
       <c r="H18" s="3">
         <v>0</v>
       </c>
-      <c r="I18" s="109">
+      <c r="I18" s="96">
         <v>34365</v>
       </c>
-      <c r="J18" s="109">
+      <c r="J18" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10294,10 +10295,10 @@
       <c r="H19" s="3">
         <v>0</v>
       </c>
-      <c r="I19" s="109">
+      <c r="I19" s="96">
         <v>30680</v>
       </c>
-      <c r="J19" s="109">
+      <c r="J19" s="96">
         <v>44925</v>
       </c>
     </row>
@@ -10331,10 +10332,10 @@
       <c r="H21" s="3">
         <v>0</v>
       </c>
-      <c r="I21" s="109">
+      <c r="I21" s="96">
         <v>28886</v>
       </c>
-      <c r="J21" s="109">
+      <c r="J21" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10363,10 +10364,10 @@
       <c r="H22" s="3">
         <v>0</v>
       </c>
-      <c r="I22" s="109">
+      <c r="I22" s="96">
         <v>28886</v>
       </c>
-      <c r="J22" s="109">
+      <c r="J22" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10395,10 +10396,10 @@
       <c r="H23" s="3">
         <v>0</v>
       </c>
-      <c r="I23" s="109">
+      <c r="I23" s="96">
         <v>28886</v>
       </c>
-      <c r="J23" s="109">
+      <c r="J23" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10427,10 +10428,10 @@
       <c r="H24" s="3">
         <v>0.7</v>
       </c>
-      <c r="I24" s="109">
+      <c r="I24" s="96">
         <v>25626</v>
       </c>
-      <c r="J24" s="109">
+      <c r="J24" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10459,10 +10460,10 @@
       <c r="H25" s="3">
         <v>0.7</v>
       </c>
-      <c r="I25" s="109">
+      <c r="I25" s="96">
         <v>25598</v>
       </c>
-      <c r="J25" s="109">
+      <c r="J25" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10491,10 +10492,10 @@
       <c r="H26" s="3">
         <v>0.7</v>
       </c>
-      <c r="I26" s="109">
+      <c r="I26" s="96">
         <v>25598</v>
       </c>
-      <c r="J26" s="109">
+      <c r="J26" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10523,10 +10524,10 @@
       <c r="H27" s="3">
         <v>0.7</v>
       </c>
-      <c r="I27" s="109">
+      <c r="I27" s="96">
         <v>25626</v>
       </c>
-      <c r="J27" s="109">
+      <c r="J27" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10555,10 +10556,10 @@
       <c r="H28" s="3">
         <v>0</v>
       </c>
-      <c r="I28" s="109">
+      <c r="I28" s="96">
         <v>32171</v>
       </c>
-      <c r="J28" s="109">
+      <c r="J28" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10587,10 +10588,10 @@
       <c r="H29" s="3">
         <v>0.7</v>
       </c>
-      <c r="I29" s="109">
+      <c r="I29" s="96">
         <v>32720</v>
       </c>
-      <c r="J29" s="109">
+      <c r="J29" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10619,10 +10620,10 @@
       <c r="H30" s="3">
         <v>0.7</v>
       </c>
-      <c r="I30" s="109">
+      <c r="I30" s="96">
         <v>36189</v>
       </c>
-      <c r="J30" s="109">
+      <c r="J30" s="96">
         <v>45777</v>
       </c>
     </row>
@@ -10646,59 +10647,59 @@
   <sheetData>
     <row r="1" spans="1:13" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4"/>
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="145" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113"/>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113"/>
-      <c r="G1" s="113"/>
-      <c r="H1" s="111"/>
-      <c r="I1" s="113" t="s">
+      <c r="C1" s="145"/>
+      <c r="D1" s="145"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="145"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="145" t="s">
         <v>168</v>
       </c>
-      <c r="J1" s="113"/>
+      <c r="J1" s="145"/>
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
     </row>
     <row r="2" spans="1:13" s="10" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A2" s="116"/>
-      <c r="B2" s="117" t="s">
+      <c r="A2" s="102"/>
+      <c r="B2" s="103" t="s">
         <v>162</v>
       </c>
-      <c r="C2" s="118" t="s">
+      <c r="C2" s="104" t="s">
         <v>163</v>
       </c>
-      <c r="D2" s="117" t="s">
+      <c r="D2" s="103" t="s">
         <v>164</v>
       </c>
-      <c r="E2" s="117" t="s">
+      <c r="E2" s="103" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="117" t="s">
+      <c r="F2" s="103" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="118" t="s">
+      <c r="G2" s="104" t="s">
         <v>165</v>
       </c>
-      <c r="H2" s="117" t="s">
+      <c r="H2" s="103" t="s">
         <v>69</v>
       </c>
-      <c r="I2" s="117" t="s">
+      <c r="I2" s="103" t="s">
         <v>166</v>
       </c>
-      <c r="J2" s="117" t="s">
+      <c r="J2" s="103" t="s">
         <v>167</v>
       </c>
-      <c r="K2" s="141" t="s">
+      <c r="K2" s="127" t="s">
         <v>169</v>
       </c>
-      <c r="L2" s="117" t="s">
+      <c r="L2" s="103" t="s">
         <v>170</v>
       </c>
-      <c r="M2" s="133" t="s">
+      <c r="M2" s="119" t="s">
         <v>171</v>
       </c>
     </row>
@@ -10706,59 +10707,59 @@
       <c r="A3" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="B3" s="112"/>
-      <c r="C3" s="112"/>
-      <c r="D3" s="112"/>
-      <c r="E3" s="112"/>
-      <c r="F3" s="114"/>
-      <c r="G3" s="112"/>
-      <c r="H3" s="112"/>
-      <c r="I3" s="119"/>
-      <c r="J3" s="119"/>
-      <c r="K3" s="142"/>
-      <c r="L3" s="134"/>
-      <c r="M3" s="135"/>
+      <c r="B3" s="99"/>
+      <c r="C3" s="99"/>
+      <c r="D3" s="99"/>
+      <c r="E3" s="99"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="99"/>
+      <c r="H3" s="99"/>
+      <c r="I3" s="105"/>
+      <c r="J3" s="105"/>
+      <c r="K3" s="128"/>
+      <c r="L3" s="120"/>
+      <c r="M3" s="121"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="112">
+      <c r="B4" s="99">
         <v>5.7241236937856403E-3</v>
       </c>
-      <c r="C4" s="112">
+      <c r="C4" s="99">
         <v>1.08524678406041E-2</v>
       </c>
-      <c r="D4" s="112">
+      <c r="D4" s="99">
         <v>1.59808119874227E-2</v>
       </c>
-      <c r="E4" s="112">
+      <c r="E4" s="99">
         <v>3.2071468696963902E-2</v>
       </c>
-      <c r="F4" s="114">
+      <c r="F4" s="100">
         <v>0.33838387456298602</v>
       </c>
-      <c r="G4" s="112">
+      <c r="G4" s="99">
         <v>3.5852467840604099E-2</v>
       </c>
-      <c r="H4" s="112">
+      <c r="H4" s="99">
         <v>0</v>
       </c>
-      <c r="I4" s="120">
+      <c r="I4" s="106">
         <v>26723</v>
       </c>
-      <c r="J4" s="120">
+      <c r="J4" s="106">
         <v>45777</v>
       </c>
-      <c r="K4" s="143">
+      <c r="K4" s="129">
         <f>Assumptions!D4</f>
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="L4" s="136">
+      <c r="L4" s="122">
         <f>C4</f>
         <v>1.08524678406041E-2</v>
       </c>
-      <c r="M4" s="137">
+      <c r="M4" s="123">
         <f>L4-K4</f>
         <v>-1.4753215939589982E-4</v>
       </c>
@@ -10767,42 +10768,42 @@
       <c r="A5" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="112">
+      <c r="B5" s="99">
         <v>4.32971260588862E-4</v>
       </c>
-      <c r="C5" s="112">
+      <c r="C5" s="99">
         <v>3.0821903711752401E-3</v>
       </c>
-      <c r="D5" s="112">
+      <c r="D5" s="99">
         <v>5.73140948176162E-3</v>
       </c>
-      <c r="E5" s="112">
+      <c r="E5" s="99">
         <v>1.4716286970652999E-2</v>
       </c>
-      <c r="F5" s="114">
+      <c r="F5" s="100">
         <v>0.20944076296702299</v>
       </c>
-      <c r="G5" s="112">
+      <c r="G5" s="99">
         <v>2.8082190371175202E-2</v>
       </c>
-      <c r="H5" s="112">
+      <c r="H5" s="99">
         <v>0</v>
       </c>
-      <c r="I5" s="120">
+      <c r="I5" s="106">
         <v>33662</v>
       </c>
-      <c r="J5" s="120">
+      <c r="J5" s="106">
         <v>45777</v>
       </c>
-      <c r="K5" s="143">
+      <c r="K5" s="129">
         <f>Assumptions!D5</f>
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="L5" s="136">
+      <c r="L5" s="122">
         <f t="shared" ref="L5:L30" si="0">C5</f>
         <v>3.0821903711752401E-3</v>
       </c>
-      <c r="M5" s="137">
+      <c r="M5" s="123">
         <f t="shared" ref="M5:M30" si="1">L5-K5</f>
         <v>-9.1780962882475996E-4</v>
       </c>
@@ -10811,59 +10812,59 @@
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="112"/>
-      <c r="C6" s="112"/>
-      <c r="D6" s="112"/>
-      <c r="E6" s="112"/>
-      <c r="F6" s="114"/>
-      <c r="G6" s="112"/>
-      <c r="H6" s="112"/>
-      <c r="I6" s="120"/>
-      <c r="J6" s="120"/>
-      <c r="K6" s="143"/>
-      <c r="L6" s="136"/>
-      <c r="M6" s="137"/>
+      <c r="B6" s="99"/>
+      <c r="C6" s="99"/>
+      <c r="D6" s="99"/>
+      <c r="E6" s="99"/>
+      <c r="F6" s="100"/>
+      <c r="G6" s="99"/>
+      <c r="H6" s="99"/>
+      <c r="I6" s="106"/>
+      <c r="J6" s="106"/>
+      <c r="K6" s="129"/>
+      <c r="L6" s="122"/>
+      <c r="M6" s="123"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="129" t="s">
+      <c r="A7" s="115" t="s">
         <v>154</v>
       </c>
-      <c r="B7" s="130">
+      <c r="B7" s="116">
         <v>2.64039774019777E-2</v>
       </c>
-      <c r="C7" s="130">
+      <c r="C7" s="116">
         <v>4.3364015406650899E-2</v>
       </c>
-      <c r="D7" s="130">
+      <c r="D7" s="116">
         <v>6.0324053411324102E-2</v>
       </c>
-      <c r="E7" s="130">
+      <c r="E7" s="116">
         <v>0.106064123700363</v>
       </c>
-      <c r="F7" s="131">
+      <c r="F7" s="117">
         <v>0.40884715673658401</v>
       </c>
-      <c r="G7" s="130">
+      <c r="G7" s="116">
         <v>6.8364015406650894E-2</v>
       </c>
-      <c r="H7" s="130">
+      <c r="H7" s="116">
         <v>0</v>
       </c>
-      <c r="I7" s="132">
+      <c r="I7" s="118">
         <v>30589</v>
       </c>
-      <c r="J7" s="132">
+      <c r="J7" s="118">
         <v>45777</v>
       </c>
-      <c r="K7" s="144">
+      <c r="K7" s="130">
         <f>Assumptions!D7</f>
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="L7" s="138">
+      <c r="L7" s="124">
         <f t="shared" si="0"/>
         <v>4.3364015406650899E-2</v>
       </c>
-      <c r="M7" s="139">
+      <c r="M7" s="125">
         <f t="shared" si="1"/>
         <v>8.3640154066508959E-3</v>
       </c>
@@ -10872,59 +10873,59 @@
       <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="112"/>
-      <c r="C8" s="112"/>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="F8" s="114"/>
-      <c r="G8" s="112"/>
-      <c r="H8" s="112"/>
-      <c r="I8" s="120"/>
-      <c r="J8" s="120"/>
-      <c r="K8" s="143"/>
-      <c r="L8" s="136"/>
-      <c r="M8" s="137"/>
+      <c r="B8" s="99"/>
+      <c r="C8" s="99"/>
+      <c r="D8" s="99"/>
+      <c r="E8" s="99"/>
+      <c r="F8" s="100"/>
+      <c r="G8" s="99"/>
+      <c r="H8" s="99"/>
+      <c r="I8" s="106"/>
+      <c r="J8" s="106"/>
+      <c r="K8" s="129"/>
+      <c r="L8" s="122"/>
+      <c r="M8" s="123"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="129" t="s">
+      <c r="A9" s="115" t="s">
         <v>140</v>
       </c>
-      <c r="B9" s="130">
+      <c r="B9" s="116">
         <v>1.7523010713942501E-2</v>
       </c>
-      <c r="C9" s="130">
+      <c r="C9" s="116">
         <v>4.4567317353041203E-2</v>
       </c>
-      <c r="D9" s="130">
+      <c r="D9" s="116">
         <v>7.1611623992139897E-2</v>
       </c>
-      <c r="E9" s="130">
+      <c r="E9" s="116">
         <v>0.16912878874266299</v>
       </c>
-      <c r="F9" s="131">
+      <c r="F9" s="117">
         <v>0.26351112477280397</v>
       </c>
-      <c r="G9" s="130">
+      <c r="G9" s="116">
         <v>6.9567317353041197E-2</v>
       </c>
-      <c r="H9" s="130">
+      <c r="H9" s="116">
         <v>0</v>
       </c>
-      <c r="I9" s="132">
+      <c r="I9" s="118">
         <v>28886</v>
       </c>
-      <c r="J9" s="132">
+      <c r="J9" s="118">
         <v>45777</v>
       </c>
-      <c r="K9" s="144">
+      <c r="K9" s="130">
         <f>Assumptions!D9</f>
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="L9" s="138">
+      <c r="L9" s="124">
         <f t="shared" si="0"/>
         <v>4.4567317353041203E-2</v>
       </c>
-      <c r="M9" s="139">
+      <c r="M9" s="125">
         <f t="shared" si="1"/>
         <v>-9.4326826469587968E-3</v>
       </c>
@@ -10933,86 +10934,86 @@
       <c r="A10" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B10" s="112">
+      <c r="B10" s="99">
         <v>3.7739774522967298E-2</v>
       </c>
-      <c r="C10" s="112">
+      <c r="C10" s="99">
         <v>6.09896272276437E-2</v>
       </c>
-      <c r="D10" s="112">
+      <c r="D10" s="99">
         <v>8.4239479932320005E-2</v>
       </c>
-      <c r="E10" s="112">
+      <c r="E10" s="99">
         <v>0.145399158457341</v>
       </c>
-      <c r="F10" s="114">
+      <c r="F10" s="100">
         <v>0.41946341281980098</v>
       </c>
-      <c r="G10" s="112">
+      <c r="G10" s="99">
         <v>8.5989627227643695E-2</v>
       </c>
-      <c r="H10" s="112">
+      <c r="H10" s="99">
         <v>0</v>
       </c>
-      <c r="I10" s="120">
+      <c r="I10" s="106">
         <v>28886</v>
       </c>
-      <c r="J10" s="120">
+      <c r="J10" s="106">
         <v>45777</v>
       </c>
-      <c r="K10" s="143">
+      <c r="K10" s="129">
         <f>Assumptions!D10</f>
         <v>0.06</v>
       </c>
-      <c r="L10" s="136">
+      <c r="L10" s="122">
         <f t="shared" si="0"/>
         <v>6.09896272276437E-2</v>
       </c>
-      <c r="M10" s="137">
+      <c r="M10" s="123">
         <f t="shared" si="1"/>
         <v>9.8962722764370237E-4</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="129" t="s">
+      <c r="A11" s="115" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="130">
+      <c r="B11" s="116">
         <v>3.9116118459153602E-2</v>
       </c>
-      <c r="C11" s="130">
+      <c r="C11" s="116">
         <v>6.9881103642633002E-2</v>
       </c>
-      <c r="D11" s="130">
+      <c r="D11" s="116">
         <v>0.10064608882611201</v>
       </c>
-      <c r="E11" s="130">
+      <c r="E11" s="116">
         <v>0.19239704493830101</v>
       </c>
-      <c r="F11" s="131">
+      <c r="F11" s="117">
         <v>0.36321297795942198</v>
       </c>
-      <c r="G11" s="130">
+      <c r="G11" s="116">
         <v>9.4881103642632997E-2</v>
       </c>
-      <c r="H11" s="130">
+      <c r="H11" s="116">
         <v>0</v>
       </c>
-      <c r="I11" s="132">
+      <c r="I11" s="118">
         <v>28886</v>
       </c>
-      <c r="J11" s="132">
+      <c r="J11" s="118">
         <v>45777</v>
       </c>
-      <c r="K11" s="144">
+      <c r="K11" s="130">
         <f>Assumptions!D11</f>
         <v>6.3E-2</v>
       </c>
-      <c r="L11" s="138">
+      <c r="L11" s="124">
         <f t="shared" si="0"/>
         <v>6.9881103642633002E-2</v>
       </c>
-      <c r="M11" s="139">
+      <c r="M11" s="125">
         <f t="shared" si="1"/>
         <v>6.8811036426330019E-3</v>
       </c>
@@ -11021,42 +11022,42 @@
       <c r="A12" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B12" s="112">
+      <c r="B12" s="99">
         <v>2.0982633206710101E-2</v>
       </c>
-      <c r="C12" s="112">
+      <c r="C12" s="99">
         <v>4.7043208728656999E-2</v>
       </c>
-      <c r="D12" s="112">
+      <c r="D12" s="99">
         <v>7.3103784250604098E-2</v>
       </c>
-      <c r="E12" s="112">
+      <c r="E12" s="99">
         <v>0.16297676367829</v>
       </c>
-      <c r="F12" s="114">
+      <c r="F12" s="100">
         <v>0.288649790724268</v>
       </c>
-      <c r="G12" s="112">
+      <c r="G12" s="99">
         <v>7.2043208728657104E-2</v>
       </c>
-      <c r="H12" s="112">
+      <c r="H12" s="99">
         <v>0.7</v>
       </c>
-      <c r="I12" s="120">
+      <c r="I12" s="106">
         <v>25626</v>
       </c>
-      <c r="J12" s="120">
+      <c r="J12" s="106">
         <v>45777</v>
       </c>
-      <c r="K12" s="143">
+      <c r="K12" s="129">
         <f>Assumptions!D12</f>
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="L12" s="136">
+      <c r="L12" s="122">
         <f t="shared" si="0"/>
         <v>4.7043208728656999E-2</v>
       </c>
-      <c r="M12" s="137">
+      <c r="M12" s="123">
         <f t="shared" si="1"/>
         <v>-9.5679127134300213E-4</v>
       </c>
@@ -11065,42 +11066,42 @@
       <c r="A13" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B13" s="112">
+      <c r="B13" s="99">
         <v>2.5237430201924101E-2</v>
       </c>
-      <c r="C13" s="112">
+      <c r="C13" s="99">
         <v>4.8975926757622301E-2</v>
       </c>
-      <c r="D13" s="112">
+      <c r="D13" s="99">
         <v>7.2714423313320495E-2</v>
       </c>
-      <c r="E13" s="112">
+      <c r="E13" s="99">
         <v>0.14845502318157899</v>
       </c>
-      <c r="F13" s="114">
+      <c r="F13" s="100">
         <v>0.32990414004192098</v>
       </c>
-      <c r="G13" s="112">
+      <c r="G13" s="99">
         <v>7.3975926757622296E-2</v>
       </c>
-      <c r="H13" s="112">
+      <c r="H13" s="99">
         <v>0.7</v>
       </c>
-      <c r="I13" s="120">
+      <c r="I13" s="106">
         <v>25598</v>
       </c>
-      <c r="J13" s="120">
+      <c r="J13" s="106">
         <v>45777</v>
       </c>
-      <c r="K13" s="143">
+      <c r="K13" s="129">
         <f>Assumptions!D13</f>
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="L13" s="136">
+      <c r="L13" s="122">
         <f t="shared" si="0"/>
         <v>4.8975926757622301E-2</v>
       </c>
-      <c r="M13" s="137">
+      <c r="M13" s="123">
         <f t="shared" si="1"/>
         <v>-2.0240732423776955E-3</v>
       </c>
@@ -11109,130 +11110,130 @@
       <c r="A14" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B14" s="112">
+      <c r="B14" s="99">
         <v>-1.15459534877681E-3</v>
       </c>
-      <c r="C14" s="112">
+      <c r="C14" s="99">
         <v>2.82523559089745E-2</v>
       </c>
-      <c r="D14" s="112">
+      <c r="D14" s="99">
         <v>5.76593071667258E-2</v>
       </c>
-      <c r="E14" s="112">
+      <c r="E14" s="99">
         <v>0.18390421737222901</v>
       </c>
-      <c r="F14" s="114">
+      <c r="F14" s="100">
         <v>0.15362538343419599</v>
       </c>
-      <c r="G14" s="112">
+      <c r="G14" s="99">
         <v>5.3252355908974501E-2</v>
       </c>
-      <c r="H14" s="112">
+      <c r="H14" s="99">
         <v>0.7</v>
       </c>
-      <c r="I14" s="120">
+      <c r="I14" s="106">
         <v>25598</v>
       </c>
-      <c r="J14" s="120">
+      <c r="J14" s="106">
         <v>45777</v>
       </c>
-      <c r="K14" s="143">
+      <c r="K14" s="129">
         <f>Assumptions!D14</f>
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="L14" s="136">
+      <c r="L14" s="122">
         <f t="shared" si="0"/>
         <v>2.82523559089745E-2</v>
       </c>
-      <c r="M14" s="137">
+      <c r="M14" s="123">
         <f t="shared" si="1"/>
         <v>2.2523559089745009E-3</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="129" t="s">
+      <c r="A15" s="115" t="s">
         <v>146</v>
       </c>
-      <c r="B15" s="130">
+      <c r="B15" s="116">
         <v>2.74370548378081E-2</v>
       </c>
-      <c r="C15" s="130">
+      <c r="C15" s="116">
         <v>5.6359980577740498E-2</v>
       </c>
-      <c r="D15" s="130">
+      <c r="D15" s="116">
         <v>8.5282906317672894E-2</v>
       </c>
-      <c r="E15" s="130">
+      <c r="E15" s="116">
         <v>0.17096972354367099</v>
       </c>
-      <c r="F15" s="131">
+      <c r="F15" s="117">
         <v>0.32964889577857998</v>
       </c>
-      <c r="G15" s="130">
+      <c r="G15" s="116">
         <v>8.1359980577740507E-2</v>
       </c>
-      <c r="H15" s="130">
+      <c r="H15" s="116">
         <v>0.7</v>
       </c>
-      <c r="I15" s="132">
+      <c r="I15" s="118">
         <v>25626</v>
       </c>
-      <c r="J15" s="132">
+      <c r="J15" s="118">
         <v>45777</v>
       </c>
-      <c r="K15" s="144">
+      <c r="K15" s="130">
         <f>Assumptions!D15</f>
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="L15" s="138">
+      <c r="L15" s="124">
         <f t="shared" si="0"/>
         <v>5.6359980577740498E-2</v>
       </c>
-      <c r="M15" s="139">
+      <c r="M15" s="125">
         <f t="shared" si="1"/>
         <v>-1.2640019422259507E-2</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="129" t="s">
+      <c r="A16" s="115" t="s">
         <v>147</v>
       </c>
-      <c r="B16" s="130">
+      <c r="B16" s="116">
         <v>3.5865028766390701E-2</v>
       </c>
-      <c r="C16" s="130">
+      <c r="C16" s="116">
         <v>7.5241692772873098E-2</v>
       </c>
-      <c r="D16" s="130">
+      <c r="D16" s="116">
         <v>0.114618356779355</v>
       </c>
-      <c r="E16" s="130">
+      <c r="E16" s="116">
         <v>0.23276405090531699</v>
       </c>
-      <c r="F16" s="131">
+      <c r="F16" s="117">
         <v>0.32325306455282199</v>
       </c>
-      <c r="G16" s="130">
+      <c r="G16" s="116">
         <v>0.100241692772873</v>
       </c>
-      <c r="H16" s="130">
+      <c r="H16" s="116">
         <v>0</v>
       </c>
-      <c r="I16" s="132">
+      <c r="I16" s="118">
         <v>32171</v>
       </c>
-      <c r="J16" s="132">
+      <c r="J16" s="118">
         <v>45777</v>
       </c>
-      <c r="K16" s="144">
+      <c r="K16" s="130">
         <f>Assumptions!D16</f>
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="L16" s="138">
+      <c r="L16" s="124">
         <f t="shared" si="0"/>
         <v>7.5241692772873098E-2</v>
       </c>
-      <c r="M16" s="139">
+      <c r="M16" s="125">
         <f t="shared" si="1"/>
         <v>-1.0758307227126895E-2</v>
       </c>
@@ -11241,42 +11242,42 @@
       <c r="A17" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="B17" s="112">
+      <c r="B17" s="99">
         <v>3.9211523567242897E-2</v>
       </c>
-      <c r="C17" s="112">
+      <c r="C17" s="99">
         <v>6.4800724140040705E-2</v>
       </c>
-      <c r="D17" s="112">
+      <c r="D17" s="99">
         <v>9.0389924712838396E-2</v>
       </c>
-      <c r="E17" s="112">
+      <c r="E17" s="99">
         <v>0.14797197236920701</v>
       </c>
-      <c r="F17" s="114">
+      <c r="F17" s="100">
         <v>0.43792566323543602</v>
       </c>
-      <c r="G17" s="112">
+      <c r="G17" s="99">
         <v>8.98007241400407E-2</v>
       </c>
-      <c r="H17" s="112">
+      <c r="H17" s="99">
         <v>0.7</v>
       </c>
-      <c r="I17" s="120">
+      <c r="I17" s="106">
         <v>32720</v>
       </c>
-      <c r="J17" s="120">
+      <c r="J17" s="106">
         <v>45777</v>
       </c>
-      <c r="K17" s="143">
+      <c r="K17" s="129">
         <f>Assumptions!D17</f>
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="L17" s="136">
+      <c r="L17" s="122">
         <f t="shared" si="0"/>
         <v>6.4800724140040705E-2</v>
       </c>
-      <c r="M17" s="137">
+      <c r="M17" s="123">
         <f t="shared" si="1"/>
         <v>3.8007241400407066E-3</v>
       </c>
@@ -11285,42 +11286,42 @@
       <c r="A18" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B18" s="112">
+      <c r="B18" s="99">
         <v>1.6403181443203799E-2</v>
       </c>
-      <c r="C18" s="112">
+      <c r="C18" s="99">
         <v>4.4976836696510598E-2</v>
       </c>
-      <c r="D18" s="112">
+      <c r="D18" s="99">
         <v>7.3550491949817401E-2</v>
       </c>
-      <c r="E18" s="112">
+      <c r="E18" s="99">
         <v>0.139789727557039</v>
       </c>
-      <c r="F18" s="114">
+      <c r="F18" s="100">
         <v>0.32174636493341902</v>
       </c>
-      <c r="G18" s="112">
+      <c r="G18" s="99">
         <v>6.99768366965106E-2</v>
       </c>
-      <c r="H18" s="112">
+      <c r="H18" s="99">
         <v>0.7</v>
       </c>
-      <c r="I18" s="120">
+      <c r="I18" s="106">
         <v>36189</v>
       </c>
-      <c r="J18" s="120">
+      <c r="J18" s="106">
         <v>45777</v>
       </c>
-      <c r="K18" s="143">
+      <c r="K18" s="129">
         <f>Assumptions!D18</f>
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="L18" s="136">
+      <c r="L18" s="122">
         <f t="shared" si="0"/>
         <v>4.4976836696510598E-2</v>
       </c>
-      <c r="M18" s="137">
+      <c r="M18" s="123">
         <f t="shared" si="1"/>
         <v>-3.0231633034894026E-3</v>
       </c>
@@ -11329,147 +11330,147 @@
       <c r="A19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="112"/>
-      <c r="C19" s="112"/>
-      <c r="D19" s="112"/>
-      <c r="E19" s="112"/>
-      <c r="F19" s="114"/>
-      <c r="G19" s="112"/>
-      <c r="H19" s="112"/>
-      <c r="I19" s="120"/>
-      <c r="J19" s="120"/>
-      <c r="K19" s="143"/>
-      <c r="L19" s="136"/>
-      <c r="M19" s="137"/>
+      <c r="B19" s="99"/>
+      <c r="C19" s="99"/>
+      <c r="D19" s="99"/>
+      <c r="E19" s="99"/>
+      <c r="F19" s="100"/>
+      <c r="G19" s="99"/>
+      <c r="H19" s="99"/>
+      <c r="I19" s="106"/>
+      <c r="J19" s="106"/>
+      <c r="K19" s="129"/>
+      <c r="L19" s="122"/>
+      <c r="M19" s="123"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B20" s="112">
+      <c r="B20" s="99">
         <v>7.6750631221554899E-3</v>
       </c>
-      <c r="C20" s="112">
+      <c r="C20" s="99">
         <v>1.9169505465816701E-2</v>
       </c>
-      <c r="D20" s="112">
+      <c r="D20" s="99">
         <v>3.0663947809477999E-2</v>
       </c>
-      <c r="E20" s="112">
+      <c r="E20" s="99">
         <v>6.1826317761391997E-2</v>
       </c>
-      <c r="F20" s="114">
+      <c r="F20" s="100">
         <v>0.31005413487178901</v>
       </c>
-      <c r="G20" s="112">
+      <c r="G20" s="99">
         <v>4.41695054658168E-2</v>
       </c>
-      <c r="H20" s="112">
+      <c r="H20" s="99">
         <v>1</v>
       </c>
-      <c r="I20" s="120">
+      <c r="I20" s="106">
         <v>34365</v>
       </c>
-      <c r="J20" s="120">
+      <c r="J20" s="106">
         <v>45777</v>
       </c>
-      <c r="K20" s="143">
+      <c r="K20" s="129">
         <f>Assumptions!D20</f>
         <v>1.9E-2</v>
       </c>
-      <c r="L20" s="136">
+      <c r="L20" s="122">
         <f t="shared" si="0"/>
         <v>1.9169505465816701E-2</v>
       </c>
-      <c r="M20" s="137">
+      <c r="M20" s="123">
         <f t="shared" si="1"/>
         <v>1.6950546581670153E-4</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="129" t="s">
+      <c r="A21" s="115" t="s">
         <v>152</v>
       </c>
-      <c r="B21" s="130">
+      <c r="B21" s="116">
         <v>4.3657888915111303E-3</v>
       </c>
-      <c r="C21" s="130">
+      <c r="C21" s="116">
         <v>2.0771382280796301E-2</v>
       </c>
-      <c r="D21" s="130">
+      <c r="D21" s="116">
         <v>3.7176975670081602E-2</v>
       </c>
-      <c r="E21" s="130">
+      <c r="E21" s="116">
         <v>8.8242421826534606E-2</v>
       </c>
-      <c r="F21" s="131">
+      <c r="F21" s="117">
         <v>0.23538998421449001</v>
       </c>
-      <c r="G21" s="130">
+      <c r="G21" s="116">
         <v>4.5771382280796302E-2</v>
       </c>
-      <c r="H21" s="130">
+      <c r="H21" s="116">
         <v>1</v>
       </c>
-      <c r="I21" s="132">
+      <c r="I21" s="118">
         <v>34365</v>
       </c>
-      <c r="J21" s="132">
+      <c r="J21" s="118">
         <v>45777</v>
       </c>
-      <c r="K21" s="144">
+      <c r="K21" s="130">
         <f>Assumptions!D21</f>
         <v>2.7E-2</v>
       </c>
-      <c r="L21" s="138">
+      <c r="L21" s="124">
         <f t="shared" si="0"/>
         <v>2.0771382280796301E-2</v>
       </c>
-      <c r="M21" s="139">
+      <c r="M21" s="125">
         <f t="shared" si="1"/>
         <v>-6.2286177192036989E-3</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A22" s="129" t="s">
+      <c r="A22" s="115" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="130">
+      <c r="B22" s="116">
         <v>3.4812134452342201E-3</v>
       </c>
-      <c r="C22" s="130">
+      <c r="C22" s="116">
         <v>1.8658048030354601E-2</v>
       </c>
-      <c r="D22" s="130">
+      <c r="D22" s="116">
         <v>3.3834882615475001E-2</v>
       </c>
-      <c r="E22" s="130">
+      <c r="E22" s="116">
         <v>8.1633172764504602E-2</v>
       </c>
-      <c r="F22" s="131">
+      <c r="F22" s="117">
         <v>0.228559633277753</v>
       </c>
-      <c r="G22" s="130">
+      <c r="G22" s="116">
         <v>4.3658048030354599E-2</v>
       </c>
-      <c r="H22" s="130">
+      <c r="H22" s="116">
         <v>1</v>
       </c>
-      <c r="I22" s="132">
+      <c r="I22" s="118">
         <v>34365</v>
       </c>
-      <c r="J22" s="132">
+      <c r="J22" s="118">
         <v>45777</v>
       </c>
-      <c r="K22" s="144">
+      <c r="K22" s="130">
         <f>Assumptions!D22</f>
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="L22" s="138">
+      <c r="L22" s="124">
         <f t="shared" si="0"/>
         <v>1.8658048030354601E-2</v>
       </c>
-      <c r="M22" s="139">
+      <c r="M22" s="125">
         <f t="shared" si="1"/>
         <v>-1.0341951969645401E-2</v>
       </c>
@@ -11478,59 +11479,59 @@
       <c r="A23" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="112"/>
-      <c r="C23" s="112"/>
-      <c r="D23" s="112"/>
-      <c r="E23" s="112"/>
-      <c r="F23" s="114"/>
-      <c r="G23" s="112"/>
-      <c r="H23" s="112"/>
-      <c r="I23" s="120"/>
-      <c r="J23" s="120"/>
-      <c r="K23" s="143"/>
-      <c r="L23" s="136"/>
-      <c r="M23" s="137"/>
+      <c r="B23" s="99"/>
+      <c r="C23" s="99"/>
+      <c r="D23" s="99"/>
+      <c r="E23" s="99"/>
+      <c r="F23" s="100"/>
+      <c r="G23" s="99"/>
+      <c r="H23" s="99"/>
+      <c r="I23" s="106"/>
+      <c r="J23" s="106"/>
+      <c r="K23" s="129"/>
+      <c r="L23" s="122"/>
+      <c r="M23" s="123"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="B24" s="112">
+      <c r="B24" s="99">
         <v>2.6608812004023499E-2</v>
       </c>
-      <c r="C24" s="112">
+      <c r="C24" s="99">
         <v>5.0216749358222103E-2</v>
       </c>
-      <c r="D24" s="112">
+      <c r="D24" s="99">
         <v>7.3824686712420803E-2</v>
       </c>
-      <c r="E24" s="112">
+      <c r="E24" s="99">
         <v>0.14763853637333799</v>
       </c>
-      <c r="F24" s="114">
+      <c r="F24" s="100">
         <v>0.340133074952987</v>
       </c>
-      <c r="G24" s="112">
+      <c r="G24" s="99">
         <v>7.5216749358222104E-2</v>
       </c>
-      <c r="H24" s="112">
+      <c r="H24" s="99">
         <v>0</v>
       </c>
-      <c r="I24" s="120">
+      <c r="I24" s="106">
         <v>25598</v>
       </c>
-      <c r="J24" s="120">
+      <c r="J24" s="106">
         <v>45777</v>
       </c>
-      <c r="K24" s="143">
+      <c r="K24" s="129">
         <f>Assumptions!D24</f>
         <v>0.08</v>
       </c>
-      <c r="L24" s="136">
+      <c r="L24" s="122">
         <f t="shared" si="0"/>
         <v>5.0216749358222103E-2</v>
       </c>
-      <c r="M24" s="137">
+      <c r="M24" s="123">
         <f t="shared" si="1"/>
         <v>-2.9783250641777899E-2</v>
       </c>
@@ -11539,42 +11540,42 @@
       <c r="A25" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="B25" s="112">
+      <c r="B25" s="99">
         <v>1.78707608365977E-2</v>
       </c>
-      <c r="C25" s="112">
+      <c r="C25" s="99">
         <v>3.5944264317563202E-2</v>
       </c>
-      <c r="D25" s="112">
+      <c r="D25" s="99">
         <v>5.40177677985288E-2</v>
       </c>
-      <c r="E25" s="112">
+      <c r="E25" s="99">
         <v>9.7213778264937697E-2</v>
       </c>
-      <c r="F25" s="114">
+      <c r="F25" s="100">
         <v>0.369744546082799</v>
       </c>
-      <c r="G25" s="112">
+      <c r="G25" s="99">
         <v>6.0944264317563203E-2</v>
       </c>
-      <c r="H25" s="112">
+      <c r="H25" s="99">
         <v>0</v>
       </c>
-      <c r="I25" s="120">
+      <c r="I25" s="106">
         <v>34365</v>
       </c>
-      <c r="J25" s="120">
+      <c r="J25" s="106">
         <v>45777</v>
       </c>
-      <c r="K25" s="143">
+      <c r="K25" s="129">
         <f>Assumptions!D25</f>
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="L25" s="136">
+      <c r="L25" s="122">
         <f t="shared" si="0"/>
         <v>3.5944264317563202E-2</v>
       </c>
-      <c r="M25" s="137">
+      <c r="M25" s="123">
         <f t="shared" si="1"/>
         <v>-4.6055735682436802E-2</v>
       </c>
@@ -11583,42 +11584,42 @@
       <c r="A26" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B26" s="112">
+      <c r="B26" s="99">
         <v>1.3852677823030299E-2</v>
       </c>
-      <c r="C26" s="112">
+      <c r="C26" s="99">
         <v>4.7598983442139302E-2</v>
       </c>
-      <c r="D26" s="112">
+      <c r="D26" s="99">
         <v>8.1345289061248299E-2</v>
       </c>
-      <c r="E26" s="112">
+      <c r="E26" s="99">
         <v>0.21081962919687999</v>
       </c>
-      <c r="F26" s="114">
+      <c r="F26" s="100">
         <v>0.225780605076804</v>
       </c>
-      <c r="G26" s="112">
+      <c r="G26" s="99">
         <v>7.2598983442139303E-2</v>
       </c>
-      <c r="H26" s="112">
+      <c r="H26" s="99">
         <v>0</v>
       </c>
-      <c r="I26" s="120">
+      <c r="I26" s="106">
         <v>30680</v>
       </c>
-      <c r="J26" s="120">
+      <c r="J26" s="106">
         <v>44925</v>
       </c>
-      <c r="K26" s="143">
+      <c r="K26" s="129">
         <f>Assumptions!D26</f>
         <v>7.2999999999999995E-2</v>
       </c>
-      <c r="L26" s="136">
+      <c r="L26" s="122">
         <f t="shared" si="0"/>
         <v>4.7598983442139302E-2</v>
       </c>
-      <c r="M26" s="137">
+      <c r="M26" s="123">
         <f t="shared" si="1"/>
         <v>-2.5401016557860694E-2</v>
       </c>
@@ -11627,147 +11628,147 @@
       <c r="A27" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="112"/>
-      <c r="C27" s="112"/>
-      <c r="D27" s="112"/>
-      <c r="E27" s="112"/>
-      <c r="F27" s="114"/>
-      <c r="G27" s="112"/>
-      <c r="H27" s="112"/>
-      <c r="I27" s="120"/>
-      <c r="J27" s="120"/>
-      <c r="K27" s="143"/>
-      <c r="L27" s="136"/>
-      <c r="M27" s="137"/>
+      <c r="B27" s="99"/>
+      <c r="C27" s="99"/>
+      <c r="D27" s="99"/>
+      <c r="E27" s="99"/>
+      <c r="F27" s="100"/>
+      <c r="G27" s="99"/>
+      <c r="H27" s="99"/>
+      <c r="I27" s="106"/>
+      <c r="J27" s="106"/>
+      <c r="K27" s="129"/>
+      <c r="L27" s="122"/>
+      <c r="M27" s="123"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B28" s="112">
+      <c r="B28" s="99">
         <v>2.64039774019777E-2</v>
       </c>
-      <c r="C28" s="112">
+      <c r="C28" s="99">
         <v>4.3364015406650899E-2</v>
       </c>
-      <c r="D28" s="112">
+      <c r="D28" s="99">
         <v>6.0324053411324102E-2</v>
       </c>
-      <c r="E28" s="112">
+      <c r="E28" s="99">
         <v>0.106064123700363</v>
       </c>
-      <c r="F28" s="114">
+      <c r="F28" s="100">
         <v>0.40884715673658401</v>
       </c>
-      <c r="G28" s="112">
+      <c r="G28" s="99">
         <v>6.8364015406650894E-2</v>
       </c>
-      <c r="H28" s="112">
+      <c r="H28" s="99">
         <v>0</v>
       </c>
-      <c r="I28" s="120">
+      <c r="I28" s="106">
         <v>30589</v>
       </c>
-      <c r="J28" s="120">
+      <c r="J28" s="106">
         <v>45777</v>
       </c>
-      <c r="K28" s="143">
+      <c r="K28" s="129">
         <f>Assumptions!D28</f>
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="L28" s="136">
+      <c r="L28" s="122">
         <f t="shared" si="0"/>
         <v>4.3364015406650899E-2</v>
       </c>
-      <c r="M28" s="137">
+      <c r="M28" s="123">
         <f t="shared" si="1"/>
         <v>-6.3598459334909818E-4</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="121" t="s">
+      <c r="A29" s="107" t="s">
         <v>156</v>
       </c>
-      <c r="B29" s="122">
+      <c r="B29" s="108">
         <v>3.9132178171297799E-2</v>
       </c>
-      <c r="C29" s="122">
+      <c r="C29" s="108">
         <v>6.2011235623535797E-2</v>
       </c>
-      <c r="D29" s="122">
+      <c r="D29" s="108">
         <v>8.4890293075773796E-2</v>
       </c>
-      <c r="E29" s="122">
+      <c r="E29" s="108">
         <v>0.143080291393996</v>
       </c>
-      <c r="F29" s="123">
+      <c r="F29" s="109">
         <v>0.43340165874262299</v>
       </c>
-      <c r="G29" s="122">
+      <c r="G29" s="108">
         <v>8.7011235623535799E-2</v>
       </c>
-      <c r="H29" s="122">
+      <c r="H29" s="108">
         <v>0</v>
       </c>
-      <c r="I29" s="124">
+      <c r="I29" s="110">
         <v>30650</v>
       </c>
-      <c r="J29" s="124">
+      <c r="J29" s="110">
         <v>44925</v>
       </c>
-      <c r="K29" s="143">
+      <c r="K29" s="129">
         <f>Assumptions!D29</f>
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="L29" s="136">
+      <c r="L29" s="122">
         <f t="shared" si="0"/>
         <v>6.2011235623535797E-2</v>
       </c>
-      <c r="M29" s="137">
+      <c r="M29" s="123">
         <f t="shared" si="1"/>
         <v>2.4011235623535798E-2</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A30" s="115" t="s">
+      <c r="A30" s="101" t="s">
         <v>157</v>
       </c>
-      <c r="B30" s="125">
+      <c r="B30" s="111">
         <v>1.3852677823030299E-2</v>
       </c>
-      <c r="C30" s="125">
+      <c r="C30" s="111">
         <v>4.7598983442139302E-2</v>
       </c>
-      <c r="D30" s="125">
+      <c r="D30" s="111">
         <v>8.1345289061248299E-2</v>
       </c>
-      <c r="E30" s="125">
+      <c r="E30" s="111">
         <v>0.21081962919687999</v>
       </c>
-      <c r="F30" s="126">
+      <c r="F30" s="112">
         <v>0.225780605076804</v>
       </c>
-      <c r="G30" s="125">
+      <c r="G30" s="111">
         <v>7.2598983442139303E-2</v>
       </c>
-      <c r="H30" s="125">
+      <c r="H30" s="111">
         <v>0</v>
       </c>
-      <c r="I30" s="127">
+      <c r="I30" s="113">
         <v>30680</v>
       </c>
-      <c r="J30" s="127">
+      <c r="J30" s="113">
         <v>44925</v>
       </c>
-      <c r="K30" s="145">
+      <c r="K30" s="131">
         <f>Assumptions!D30</f>
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="L30" s="128">
+      <c r="L30" s="114">
         <f t="shared" si="0"/>
         <v>4.7598983442139302E-2</v>
       </c>
-      <c r="M30" s="140">
+      <c r="M30" s="126">
         <f t="shared" si="1"/>
         <v>4.5989834421393053E-3</v>
       </c>

</xml_diff>

<commit_message>
Reporting function for formatting assumptions, Adjust beta assumption in private assets
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/python/epsilonPhi/core/reporting/formatted_excel.xlsx
+++ b/epsilon-phi-core/src/python/epsilonPhi/core/reporting/formatted_excel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/python/epsilonPhi/core/reporting/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/python/epsilonPhi/core/reporting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C773E2-BA42-D345-A983-3571AF531347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1D610B-1983-D244-AD5C-3DF7C844BB05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="7120" windowWidth="33600" windowHeight="19040" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="26440" windowHeight="19040" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolios" sheetId="2" r:id="rId1"/>
@@ -908,7 +908,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -1081,6 +1081,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color rgb="FF737373"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1089,7 +1098,7 @@
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="206">
+  <cellXfs count="216">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1499,56 +1508,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1560,9 +1524,6 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="24" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1645,6 +1606,82 @@
     </xf>
     <xf numFmtId="17" fontId="23" fillId="16" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="11" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="24" fillId="16" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="16" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="16" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="24" fillId="16" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="24" fillId="16" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="24" fillId="16" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1667,6 +1704,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF737373"/>
       <color rgb="FF807C80"/>
       <color rgb="FF000004"/>
       <color rgb="FF039644"/>
@@ -1676,7 +1714,6 @@
       <color rgb="FF567707"/>
       <color rgb="FF0F2442"/>
       <color rgb="FFFFFFFF"/>
-      <color rgb="FFFAFFFF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -3623,107 +3660,107 @@
     <col min="9" max="10" width="11.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="169"/>
-      <c r="B1" s="170" t="s">
+    <row r="1" spans="1:10" s="8" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="213"/>
+      <c r="B1" s="214" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="170"/>
-      <c r="D1" s="170"/>
-      <c r="E1" s="170"/>
-      <c r="F1" s="170"/>
-      <c r="G1" s="170"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="170" t="s">
+      <c r="C1" s="214"/>
+      <c r="D1" s="214"/>
+      <c r="E1" s="214"/>
+      <c r="F1" s="214"/>
+      <c r="G1" s="214"/>
+      <c r="H1" s="215"/>
+      <c r="I1" s="214" t="s">
         <v>155</v>
       </c>
-      <c r="J1" s="170"/>
-    </row>
-    <row r="2" spans="1:10" s="8" customFormat="1" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="172"/>
-      <c r="B2" s="173" t="s">
+      <c r="J1" s="214"/>
+    </row>
+    <row r="2" spans="1:10" s="8" customFormat="1" ht="49" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="157"/>
+      <c r="B2" s="204" t="s">
         <v>171</v>
       </c>
-      <c r="C2" s="173"/>
-      <c r="D2" s="173"/>
-      <c r="E2" s="174" t="s">
+      <c r="C2" s="204"/>
+      <c r="D2" s="204"/>
+      <c r="E2" s="159" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="174" t="s">
+      <c r="F2" s="159" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="175" t="s">
+      <c r="G2" s="158" t="s">
         <v>152</v>
       </c>
-      <c r="H2" s="174" t="s">
+      <c r="H2" s="159" t="s">
         <v>67</v>
       </c>
-      <c r="I2" s="174" t="s">
+      <c r="I2" s="159" t="s">
         <v>153</v>
       </c>
-      <c r="J2" s="174" t="s">
+      <c r="J2" s="159" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="176" t="s">
+    <row r="3" spans="1:10" s="154" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="160" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="177"/>
-      <c r="C3" s="177"/>
-      <c r="D3" s="177"/>
-      <c r="E3" s="177"/>
-      <c r="F3" s="177"/>
-      <c r="G3" s="177"/>
-      <c r="H3" s="177"/>
-      <c r="I3" s="177"/>
-      <c r="J3" s="177"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="169" t="s">
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+    </row>
+    <row r="4" spans="1:10" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="155" t="s">
         <v>172</v>
       </c>
-      <c r="B4" s="178">
+      <c r="B4" s="162">
         <v>5.7241236937856403E-3</v>
       </c>
-      <c r="C4" s="179">
+      <c r="C4" s="163">
         <v>1.08524678406041E-2</v>
       </c>
-      <c r="D4" s="180">
+      <c r="D4" s="164">
         <v>1.59808119874227E-2</v>
       </c>
-      <c r="E4" s="179">
+      <c r="E4" s="163">
         <v>3.2071468696963902E-2</v>
       </c>
-      <c r="F4" s="181">
+      <c r="F4" s="165">
         <v>0.33838387456298602</v>
       </c>
-      <c r="G4" s="179">
+      <c r="G4" s="163">
         <v>3.5852467840604099E-2</v>
       </c>
-      <c r="H4" s="182">
+      <c r="H4" s="166">
         <v>0</v>
       </c>
-      <c r="I4" s="183">
+      <c r="I4" s="167">
         <v>26723</v>
       </c>
-      <c r="J4" s="183">
+      <c r="J4" s="167">
         <v>45777</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="192" t="s">
+    <row r="5" spans="1:10" s="154" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="206" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="193"/>
-      <c r="C5" s="194"/>
-      <c r="D5" s="195"/>
-      <c r="E5" s="194"/>
-      <c r="F5" s="196"/>
-      <c r="G5" s="194"/>
-      <c r="H5" s="197"/>
-      <c r="I5" s="198"/>
-      <c r="J5" s="198"/>
+      <c r="B5" s="207"/>
+      <c r="C5" s="208"/>
+      <c r="D5" s="209"/>
+      <c r="E5" s="208"/>
+      <c r="F5" s="210"/>
+      <c r="G5" s="208"/>
+      <c r="H5" s="211"/>
+      <c r="I5" s="212"/>
+      <c r="J5" s="212"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3835,232 +3872,232 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="53"/>
-      <c r="B1" s="160" t="s">
+      <c r="B1" s="197" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160" t="s">
+      <c r="C1" s="197"/>
+      <c r="D1" s="197" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160" t="s">
+      <c r="E1" s="197"/>
+      <c r="F1" s="197" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160" t="s">
+      <c r="G1" s="197"/>
+      <c r="H1" s="197" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="161"/>
+      <c r="I1" s="198"/>
     </row>
     <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="162">
+      <c r="B2" s="199">
         <v>0.745</v>
       </c>
-      <c r="C2" s="162"/>
-      <c r="D2" s="162" t="s">
+      <c r="C2" s="199"/>
+      <c r="D2" s="199" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="162"/>
-      <c r="F2" s="162">
+      <c r="E2" s="199"/>
+      <c r="F2" s="199">
         <v>0.36</v>
       </c>
-      <c r="G2" s="162"/>
-      <c r="H2" s="162">
+      <c r="G2" s="199"/>
+      <c r="H2" s="199">
         <v>0.15</v>
       </c>
-      <c r="I2" s="162"/>
+      <c r="I2" s="199"/>
     </row>
     <row r="3" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="155">
+      <c r="B3" s="192">
         <v>0.02</v>
       </c>
-      <c r="C3" s="155"/>
-      <c r="D3" s="155">
+      <c r="C3" s="192"/>
+      <c r="D3" s="192">
         <v>0.03</v>
       </c>
-      <c r="E3" s="155"/>
-      <c r="F3" s="155">
+      <c r="E3" s="192"/>
+      <c r="F3" s="192">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155">
+      <c r="G3" s="192"/>
+      <c r="H3" s="192">
         <v>5.5E-2</v>
       </c>
-      <c r="I3" s="155"/>
+      <c r="I3" s="192"/>
     </row>
     <row r="4" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="155">
+      <c r="B4" s="192">
         <v>0.14000000000000001</v>
       </c>
-      <c r="C4" s="155"/>
-      <c r="D4" s="155">
+      <c r="C4" s="192"/>
+      <c r="D4" s="192">
         <v>0.22500000000000001</v>
       </c>
-      <c r="E4" s="155"/>
-      <c r="F4" s="155">
+      <c r="E4" s="192"/>
+      <c r="F4" s="192">
         <v>0.35499999999999998</v>
       </c>
-      <c r="G4" s="155"/>
-      <c r="H4" s="155">
+      <c r="G4" s="192"/>
+      <c r="H4" s="192">
         <v>0.505</v>
       </c>
-      <c r="I4" s="155"/>
+      <c r="I4" s="192"/>
     </row>
     <row r="5" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="155">
+      <c r="B5" s="192">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C5" s="155"/>
-      <c r="D5" s="155">
+      <c r="C5" s="192"/>
+      <c r="D5" s="192">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E5" s="155"/>
-      <c r="F5" s="155">
+      <c r="E5" s="192"/>
+      <c r="F5" s="192">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G5" s="155"/>
-      <c r="H5" s="155">
+      <c r="G5" s="192"/>
+      <c r="H5" s="192">
         <v>0.03</v>
       </c>
-      <c r="I5" s="155"/>
+      <c r="I5" s="192"/>
     </row>
     <row r="6" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="155">
+      <c r="B6" s="192">
         <v>0.04</v>
       </c>
-      <c r="C6" s="155"/>
-      <c r="D6" s="155">
+      <c r="C6" s="192"/>
+      <c r="D6" s="192">
         <v>5.5E-2</v>
       </c>
-      <c r="E6" s="155"/>
-      <c r="F6" s="155">
+      <c r="E6" s="192"/>
+      <c r="F6" s="192">
         <v>0.12</v>
       </c>
-      <c r="G6" s="155"/>
-      <c r="H6" s="155">
+      <c r="G6" s="192"/>
+      <c r="H6" s="192">
         <v>0.185</v>
       </c>
-      <c r="I6" s="155"/>
+      <c r="I6" s="192"/>
     </row>
     <row r="7" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="156">
+      <c r="B7" s="193">
         <v>0.04</v>
       </c>
-      <c r="C7" s="156"/>
-      <c r="D7" s="156">
+      <c r="C7" s="193"/>
+      <c r="D7" s="193">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E7" s="156"/>
-      <c r="F7" s="156">
+      <c r="E7" s="193"/>
+      <c r="F7" s="193">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G7" s="156"/>
-      <c r="H7" s="156">
+      <c r="G7" s="193"/>
+      <c r="H7" s="193">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I7" s="156"/>
+      <c r="I7" s="193"/>
     </row>
     <row r="8" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="157">
+      <c r="B8" s="194">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="C8" s="157"/>
-      <c r="D8" s="157">
+      <c r="C8" s="194"/>
+      <c r="D8" s="194">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E8" s="157"/>
-      <c r="F8" s="157">
+      <c r="E8" s="194"/>
+      <c r="F8" s="194">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G8" s="157"/>
-      <c r="H8" s="157">
+      <c r="G8" s="194"/>
+      <c r="H8" s="194">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="I8" s="157"/>
+      <c r="I8" s="194"/>
     </row>
     <row r="9" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="58" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="158">
+      <c r="B9" s="195">
         <v>0.6</v>
       </c>
-      <c r="C9" s="158"/>
-      <c r="D9" s="158">
+      <c r="C9" s="195"/>
+      <c r="D9" s="195">
         <v>0.59</v>
       </c>
-      <c r="E9" s="158"/>
-      <c r="F9" s="158">
+      <c r="E9" s="195"/>
+      <c r="F9" s="195">
         <v>0.53</v>
       </c>
-      <c r="G9" s="158"/>
-      <c r="H9" s="158">
+      <c r="G9" s="195"/>
+      <c r="H9" s="195">
         <v>0.49</v>
       </c>
-      <c r="I9" s="158"/>
+      <c r="I9" s="195"/>
     </row>
     <row r="10" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="155">
+      <c r="B10" s="192">
         <v>3.1E-2</v>
       </c>
-      <c r="C10" s="155"/>
-      <c r="D10" s="155">
+      <c r="C10" s="192"/>
+      <c r="D10" s="192">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="E10" s="155"/>
-      <c r="F10" s="155">
+      <c r="E10" s="192"/>
+      <c r="F10" s="192">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="G10" s="155"/>
-      <c r="H10" s="155">
+      <c r="G10" s="192"/>
+      <c r="H10" s="192">
         <v>0.10299999999999999</v>
       </c>
-      <c r="I10" s="155"/>
+      <c r="I10" s="192"/>
     </row>
     <row r="11" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="159" t="s">
+      <c r="B11" s="196" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="159"/>
-      <c r="D11" s="159" t="s">
+      <c r="C11" s="196"/>
+      <c r="D11" s="196" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="159"/>
-      <c r="F11" s="159" t="s">
+      <c r="E11" s="196"/>
+      <c r="F11" s="196" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="159"/>
-      <c r="H11" s="159" t="s">
+      <c r="G11" s="196"/>
+      <c r="H11" s="196" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="159"/>
+      <c r="I11" s="196"/>
     </row>
     <row r="12" spans="1:9" s="8" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="59" t="s">
@@ -4353,64 +4390,64 @@
       <c r="A23" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="153">
+      <c r="B23" s="190">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="C23" s="153"/>
-      <c r="D23" s="153">
+      <c r="C23" s="190"/>
+      <c r="D23" s="190">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="E23" s="153"/>
-      <c r="F23" s="153">
+      <c r="E23" s="190"/>
+      <c r="F23" s="190">
         <v>6.3E-2</v>
       </c>
-      <c r="G23" s="153"/>
-      <c r="H23" s="153">
+      <c r="G23" s="190"/>
+      <c r="H23" s="190">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="I23" s="153"/>
+      <c r="I23" s="190"/>
     </row>
     <row r="24" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="62" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="153">
+      <c r="B24" s="190">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C24" s="153"/>
-      <c r="D24" s="153">
+      <c r="C24" s="190"/>
+      <c r="D24" s="190">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="E24" s="153"/>
-      <c r="F24" s="153">
+      <c r="E24" s="190"/>
+      <c r="F24" s="190">
         <v>0.16200000000000001</v>
       </c>
-      <c r="G24" s="153"/>
-      <c r="H24" s="153">
+      <c r="G24" s="190"/>
+      <c r="H24" s="190">
         <v>0.24299999999999999</v>
       </c>
-      <c r="I24" s="153"/>
+      <c r="I24" s="190"/>
     </row>
     <row r="25" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="154">
+      <c r="B25" s="191">
         <v>0</v>
       </c>
-      <c r="C25" s="154"/>
-      <c r="D25" s="154">
+      <c r="C25" s="191"/>
+      <c r="D25" s="191">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="E25" s="154"/>
-      <c r="F25" s="154">
+      <c r="E25" s="191"/>
+      <c r="F25" s="191">
         <v>0.14899999999999999</v>
       </c>
-      <c r="G25" s="154"/>
-      <c r="H25" s="154">
+      <c r="G25" s="191"/>
+      <c r="H25" s="191">
         <v>0.253</v>
       </c>
-      <c r="I25" s="154"/>
+      <c r="I25" s="191"/>
     </row>
     <row r="26" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="67" t="s">
@@ -4429,64 +4466,64 @@
       <c r="A27" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="153">
+      <c r="B27" s="190">
         <v>0.23799999999999999</v>
       </c>
-      <c r="C27" s="153"/>
-      <c r="D27" s="153">
+      <c r="C27" s="190"/>
+      <c r="D27" s="190">
         <v>0.27900000000000003</v>
       </c>
-      <c r="E27" s="153"/>
-      <c r="F27" s="153">
+      <c r="E27" s="190"/>
+      <c r="F27" s="190">
         <v>0.314</v>
       </c>
-      <c r="G27" s="153"/>
-      <c r="H27" s="153">
+      <c r="G27" s="190"/>
+      <c r="H27" s="190">
         <v>0.33700000000000002</v>
       </c>
-      <c r="I27" s="153"/>
+      <c r="I27" s="190"/>
     </row>
     <row r="28" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="62" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="153">
+      <c r="B28" s="190">
         <v>0.04</v>
       </c>
-      <c r="C28" s="153"/>
-      <c r="D28" s="153">
+      <c r="C28" s="190"/>
+      <c r="D28" s="190">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="E28" s="153"/>
-      <c r="F28" s="153">
+      <c r="E28" s="190"/>
+      <c r="F28" s="190">
         <v>0.14299999999999999</v>
       </c>
-      <c r="G28" s="153"/>
-      <c r="H28" s="153">
+      <c r="G28" s="190"/>
+      <c r="H28" s="190">
         <v>0.187</v>
       </c>
-      <c r="I28" s="153"/>
+      <c r="I28" s="190"/>
     </row>
     <row r="29" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="153">
+      <c r="B29" s="190">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C29" s="153"/>
-      <c r="D29" s="153">
+      <c r="C29" s="190"/>
+      <c r="D29" s="190">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="E29" s="153"/>
-      <c r="F29" s="153">
+      <c r="E29" s="190"/>
+      <c r="F29" s="190">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G29" s="153"/>
-      <c r="H29" s="153">
+      <c r="G29" s="190"/>
+      <c r="H29" s="190">
         <v>0.108</v>
       </c>
-      <c r="I29" s="153"/>
+      <c r="I29" s="190"/>
     </row>
     <row r="30" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="59" t="s">
@@ -5131,16 +5168,16 @@
   <sheetData>
     <row r="1" spans="1:16" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="19"/>
-      <c r="B1" s="165" t="s">
+      <c r="B1" s="202" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="165"/>
-      <c r="D1" s="165"/>
-      <c r="E1" s="165"/>
-      <c r="F1" s="165"/>
-      <c r="G1" s="165"/>
-      <c r="H1" s="165"/>
-      <c r="I1" s="165"/>
+      <c r="C1" s="202"/>
+      <c r="D1" s="202"/>
+      <c r="E1" s="202"/>
+      <c r="F1" s="202"/>
+      <c r="G1" s="202"/>
+      <c r="H1" s="202"/>
+      <c r="I1" s="202"/>
       <c r="J1" s="21"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
@@ -5148,13 +5185,13 @@
     </row>
     <row r="2" spans="1:16" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="22"/>
-      <c r="B2" s="163" t="s">
+      <c r="B2" s="200" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="163"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="164"/>
+      <c r="C2" s="200"/>
+      <c r="D2" s="201"/>
+      <c r="E2" s="201"/>
+      <c r="F2" s="201"/>
       <c r="G2" s="24" t="s">
         <v>31</v>
       </c>
@@ -6016,7 +6053,7 @@
       <c r="P26" s="3"/>
     </row>
     <row r="27" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="167" t="s">
+      <c r="A27" s="153" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="30"/>
@@ -6302,832 +6339,832 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="169"/>
-      <c r="B1" s="170" t="s">
+      <c r="A1" s="155"/>
+      <c r="B1" s="203" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="170"/>
-      <c r="D1" s="170"/>
-      <c r="E1" s="170"/>
-      <c r="F1" s="170"/>
-      <c r="G1" s="170"/>
-      <c r="H1" s="171"/>
-      <c r="I1" s="170" t="s">
+      <c r="C1" s="203"/>
+      <c r="D1" s="203"/>
+      <c r="E1" s="203"/>
+      <c r="F1" s="203"/>
+      <c r="G1" s="203"/>
+      <c r="H1" s="156"/>
+      <c r="I1" s="203" t="s">
         <v>155</v>
       </c>
-      <c r="J1" s="170"/>
+      <c r="J1" s="203"/>
     </row>
     <row r="2" spans="1:10" s="8" customFormat="1" ht="46" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="172"/>
-      <c r="B2" s="173" t="s">
+      <c r="A2" s="157"/>
+      <c r="B2" s="204" t="s">
         <v>171</v>
       </c>
-      <c r="C2" s="173"/>
-      <c r="D2" s="173"/>
-      <c r="E2" s="174" t="s">
+      <c r="C2" s="204"/>
+      <c r="D2" s="204"/>
+      <c r="E2" s="159" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="174" t="s">
+      <c r="F2" s="159" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="175" t="s">
+      <c r="G2" s="158" t="s">
         <v>152</v>
       </c>
-      <c r="H2" s="174" t="s">
+      <c r="H2" s="159" t="s">
         <v>67</v>
       </c>
-      <c r="I2" s="174" t="s">
+      <c r="I2" s="159" t="s">
         <v>153</v>
       </c>
-      <c r="J2" s="174" t="s">
+      <c r="J2" s="159" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="176" t="s">
+    <row r="3" spans="1:10" s="154" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="160" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="177"/>
-      <c r="C3" s="177"/>
-      <c r="D3" s="177"/>
-      <c r="E3" s="177"/>
-      <c r="F3" s="177"/>
-      <c r="G3" s="177"/>
-      <c r="H3" s="177"/>
-      <c r="I3" s="177"/>
-      <c r="J3" s="177"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="169" t="s">
+      <c r="A4" s="155" t="s">
         <v>172</v>
       </c>
-      <c r="B4" s="178">
+      <c r="B4" s="162">
         <v>5.7241236937856403E-3</v>
       </c>
-      <c r="C4" s="179">
+      <c r="C4" s="163">
         <v>1.08524678406041E-2</v>
       </c>
-      <c r="D4" s="180">
+      <c r="D4" s="164">
         <v>1.59808119874227E-2</v>
       </c>
-      <c r="E4" s="179">
+      <c r="E4" s="163">
         <v>3.2071468696963902E-2</v>
       </c>
-      <c r="F4" s="181">
+      <c r="F4" s="165">
         <v>0.33838387456298602</v>
       </c>
-      <c r="G4" s="179">
+      <c r="G4" s="163">
         <v>3.5852467840604099E-2</v>
       </c>
-      <c r="H4" s="182">
+      <c r="H4" s="166">
         <v>0</v>
       </c>
-      <c r="I4" s="183">
+      <c r="I4" s="167">
         <v>26723</v>
       </c>
-      <c r="J4" s="183">
+      <c r="J4" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="199" t="s">
+      <c r="A5" s="183" t="s">
         <v>173</v>
       </c>
-      <c r="B5" s="200">
+      <c r="B5" s="184">
         <v>4.32971260588862E-4</v>
       </c>
-      <c r="C5" s="201">
+      <c r="C5" s="185">
         <v>3.0821903711752401E-3</v>
       </c>
-      <c r="D5" s="202">
+      <c r="D5" s="186">
         <v>5.73140948176162E-3</v>
       </c>
-      <c r="E5" s="201">
+      <c r="E5" s="185">
         <v>1.4716286970652999E-2</v>
       </c>
-      <c r="F5" s="203">
+      <c r="F5" s="187">
         <v>0.20944076296702299</v>
       </c>
-      <c r="G5" s="201">
+      <c r="G5" s="185">
         <v>2.8082190371175202E-2</v>
       </c>
-      <c r="H5" s="204">
+      <c r="H5" s="188">
         <v>0</v>
       </c>
-      <c r="I5" s="205">
+      <c r="I5" s="189">
         <v>33662</v>
       </c>
-      <c r="J5" s="205">
+      <c r="J5" s="189">
         <v>45777</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="192" t="s">
+    <row r="6" spans="1:10" s="154" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="193"/>
-      <c r="C6" s="194"/>
-      <c r="D6" s="195"/>
-      <c r="E6" s="194"/>
-      <c r="F6" s="196"/>
-      <c r="G6" s="194"/>
-      <c r="H6" s="197"/>
-      <c r="I6" s="198"/>
-      <c r="J6" s="198"/>
+      <c r="B6" s="177"/>
+      <c r="C6" s="178"/>
+      <c r="D6" s="179"/>
+      <c r="E6" s="178"/>
+      <c r="F6" s="180"/>
+      <c r="G6" s="178"/>
+      <c r="H6" s="181"/>
+      <c r="I6" s="182"/>
+      <c r="J6" s="182"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="199" t="s">
+      <c r="A7" s="183" t="s">
         <v>174</v>
       </c>
-      <c r="B7" s="200">
+      <c r="B7" s="184">
         <v>2.64039774019777E-2</v>
       </c>
-      <c r="C7" s="201">
+      <c r="C7" s="185">
         <v>4.3364015406650899E-2</v>
       </c>
-      <c r="D7" s="202">
+      <c r="D7" s="186">
         <v>6.0324053411324102E-2</v>
       </c>
-      <c r="E7" s="201">
+      <c r="E7" s="185">
         <v>0.106064123700363</v>
       </c>
-      <c r="F7" s="203">
+      <c r="F7" s="187">
         <v>0.40884715673658401</v>
       </c>
-      <c r="G7" s="201">
+      <c r="G7" s="185">
         <v>6.8364015406650894E-2</v>
       </c>
-      <c r="H7" s="204">
+      <c r="H7" s="188">
         <v>0</v>
       </c>
-      <c r="I7" s="205">
+      <c r="I7" s="189">
         <v>30589</v>
       </c>
-      <c r="J7" s="205">
+      <c r="J7" s="189">
         <v>45777</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="192" t="s">
+    <row r="8" spans="1:10" s="154" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="176" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="193"/>
-      <c r="C8" s="194"/>
-      <c r="D8" s="195"/>
-      <c r="E8" s="194"/>
-      <c r="F8" s="196"/>
-      <c r="G8" s="194"/>
-      <c r="H8" s="197"/>
-      <c r="I8" s="198"/>
-      <c r="J8" s="198"/>
+      <c r="B8" s="177"/>
+      <c r="C8" s="178"/>
+      <c r="D8" s="179"/>
+      <c r="E8" s="178"/>
+      <c r="F8" s="180"/>
+      <c r="G8" s="178"/>
+      <c r="H8" s="181"/>
+      <c r="I8" s="182"/>
+      <c r="J8" s="182"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="169" t="s">
+      <c r="A9" s="155" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="178">
+      <c r="B9" s="162">
         <v>1.7523010713942501E-2</v>
       </c>
-      <c r="C9" s="179">
+      <c r="C9" s="163">
         <v>4.4567317353041203E-2</v>
       </c>
-      <c r="D9" s="180">
+      <c r="D9" s="164">
         <v>7.1611623992139897E-2</v>
       </c>
-      <c r="E9" s="179">
+      <c r="E9" s="163">
         <v>0.16912878874266299</v>
       </c>
-      <c r="F9" s="181">
+      <c r="F9" s="165">
         <v>0.26351112477280397</v>
       </c>
-      <c r="G9" s="179">
+      <c r="G9" s="163">
         <v>6.9567317353041197E-2</v>
       </c>
-      <c r="H9" s="182">
+      <c r="H9" s="166">
         <v>0</v>
       </c>
-      <c r="I9" s="183">
+      <c r="I9" s="167">
         <v>28886</v>
       </c>
-      <c r="J9" s="183">
+      <c r="J9" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="169" t="s">
+      <c r="A10" s="155" t="s">
         <v>176</v>
       </c>
-      <c r="B10" s="178">
+      <c r="B10" s="162">
         <v>3.7739774522967298E-2</v>
       </c>
-      <c r="C10" s="179">
+      <c r="C10" s="163">
         <v>6.09896272276437E-2</v>
       </c>
-      <c r="D10" s="180">
+      <c r="D10" s="164">
         <v>8.4239479932320005E-2</v>
       </c>
-      <c r="E10" s="179">
+      <c r="E10" s="163">
         <v>0.145399158457341</v>
       </c>
-      <c r="F10" s="181">
+      <c r="F10" s="165">
         <v>0.41946341281980098</v>
       </c>
-      <c r="G10" s="179">
+      <c r="G10" s="163">
         <v>8.5989627227643695E-2</v>
       </c>
-      <c r="H10" s="182">
+      <c r="H10" s="166">
         <v>0</v>
       </c>
-      <c r="I10" s="183">
+      <c r="I10" s="167">
         <v>28886</v>
       </c>
-      <c r="J10" s="183">
+      <c r="J10" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="169" t="s">
+      <c r="A11" s="155" t="s">
         <v>177</v>
       </c>
-      <c r="B11" s="178">
+      <c r="B11" s="162">
         <v>3.9116118459153602E-2</v>
       </c>
-      <c r="C11" s="179">
+      <c r="C11" s="163">
         <v>6.9881103642633002E-2</v>
       </c>
-      <c r="D11" s="180">
+      <c r="D11" s="164">
         <v>0.10064608882611201</v>
       </c>
-      <c r="E11" s="179">
+      <c r="E11" s="163">
         <v>0.19239704493830101</v>
       </c>
-      <c r="F11" s="181">
+      <c r="F11" s="165">
         <v>0.36321297795942198</v>
       </c>
-      <c r="G11" s="179">
+      <c r="G11" s="163">
         <v>9.4881103642632997E-2</v>
       </c>
-      <c r="H11" s="182">
+      <c r="H11" s="166">
         <v>0</v>
       </c>
-      <c r="I11" s="183">
+      <c r="I11" s="167">
         <v>28886</v>
       </c>
-      <c r="J11" s="183">
+      <c r="J11" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="169" t="s">
+      <c r="A12" s="155" t="s">
         <v>178</v>
       </c>
-      <c r="B12" s="178">
+      <c r="B12" s="162">
         <v>2.0982633206710101E-2</v>
       </c>
-      <c r="C12" s="179">
+      <c r="C12" s="163">
         <v>4.7043208728656999E-2</v>
       </c>
-      <c r="D12" s="180">
+      <c r="D12" s="164">
         <v>7.3103784250604098E-2</v>
       </c>
-      <c r="E12" s="179">
+      <c r="E12" s="163">
         <v>0.16297676367829</v>
       </c>
-      <c r="F12" s="181">
+      <c r="F12" s="165">
         <v>0.288649790724268</v>
       </c>
-      <c r="G12" s="179">
+      <c r="G12" s="163">
         <v>7.2043208728657104E-2</v>
       </c>
-      <c r="H12" s="182">
+      <c r="H12" s="166">
         <v>0.7</v>
       </c>
-      <c r="I12" s="183">
+      <c r="I12" s="167">
         <v>25626</v>
       </c>
-      <c r="J12" s="183">
+      <c r="J12" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="169" t="s">
+      <c r="A13" s="155" t="s">
         <v>179</v>
       </c>
-      <c r="B13" s="178">
+      <c r="B13" s="162">
         <v>2.5237430201924101E-2</v>
       </c>
-      <c r="C13" s="179">
+      <c r="C13" s="163">
         <v>4.8975926757622301E-2</v>
       </c>
-      <c r="D13" s="180">
+      <c r="D13" s="164">
         <v>7.2714423313320495E-2</v>
       </c>
-      <c r="E13" s="179">
+      <c r="E13" s="163">
         <v>0.14845502318157899</v>
       </c>
-      <c r="F13" s="181">
+      <c r="F13" s="165">
         <v>0.32990414004192098</v>
       </c>
-      <c r="G13" s="179">
+      <c r="G13" s="163">
         <v>7.3975926757622296E-2</v>
       </c>
-      <c r="H13" s="182">
+      <c r="H13" s="166">
         <v>0.7</v>
       </c>
-      <c r="I13" s="183">
+      <c r="I13" s="167">
         <v>25598</v>
       </c>
-      <c r="J13" s="183">
+      <c r="J13" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="169" t="s">
+      <c r="A14" s="155" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="178">
+      <c r="B14" s="162">
         <v>-1.15459534877681E-3</v>
       </c>
-      <c r="C14" s="179">
+      <c r="C14" s="163">
         <v>2.82523559089745E-2</v>
       </c>
-      <c r="D14" s="180">
+      <c r="D14" s="164">
         <v>5.76593071667258E-2</v>
       </c>
-      <c r="E14" s="179">
+      <c r="E14" s="163">
         <v>0.18390421737222901</v>
       </c>
-      <c r="F14" s="181">
+      <c r="F14" s="165">
         <v>0.15362538343419599</v>
       </c>
-      <c r="G14" s="179">
+      <c r="G14" s="163">
         <v>5.3252355908974501E-2</v>
       </c>
-      <c r="H14" s="182">
+      <c r="H14" s="166">
         <v>0.7</v>
       </c>
-      <c r="I14" s="183">
+      <c r="I14" s="167">
         <v>25598</v>
       </c>
-      <c r="J14" s="183">
+      <c r="J14" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="169" t="s">
+      <c r="A15" s="155" t="s">
         <v>181</v>
       </c>
-      <c r="B15" s="178">
+      <c r="B15" s="162">
         <v>2.74370548378081E-2</v>
       </c>
-      <c r="C15" s="179">
+      <c r="C15" s="163">
         <v>5.6359980577740498E-2</v>
       </c>
-      <c r="D15" s="180">
+      <c r="D15" s="164">
         <v>8.5282906317672894E-2</v>
       </c>
-      <c r="E15" s="179">
+      <c r="E15" s="163">
         <v>0.17096972354367099</v>
       </c>
-      <c r="F15" s="181">
+      <c r="F15" s="165">
         <v>0.32964889577857998</v>
       </c>
-      <c r="G15" s="179">
+      <c r="G15" s="163">
         <v>8.1359980577740507E-2</v>
       </c>
-      <c r="H15" s="182">
+      <c r="H15" s="166">
         <v>0.7</v>
       </c>
-      <c r="I15" s="183">
+      <c r="I15" s="167">
         <v>25626</v>
       </c>
-      <c r="J15" s="183">
+      <c r="J15" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="169" t="s">
+      <c r="A16" s="155" t="s">
         <v>182</v>
       </c>
-      <c r="B16" s="178">
+      <c r="B16" s="162">
         <v>3.5865028766390701E-2</v>
       </c>
-      <c r="C16" s="179">
+      <c r="C16" s="163">
         <v>7.5241692772873098E-2</v>
       </c>
-      <c r="D16" s="180">
+      <c r="D16" s="164">
         <v>0.114618356779355</v>
       </c>
-      <c r="E16" s="179">
+      <c r="E16" s="163">
         <v>0.23276405090531699</v>
       </c>
-      <c r="F16" s="181">
+      <c r="F16" s="165">
         <v>0.32325306455282199</v>
       </c>
-      <c r="G16" s="179">
+      <c r="G16" s="163">
         <v>0.100241692772873</v>
       </c>
-      <c r="H16" s="182">
+      <c r="H16" s="166">
         <v>0</v>
       </c>
-      <c r="I16" s="183">
+      <c r="I16" s="167">
         <v>32171</v>
       </c>
-      <c r="J16" s="183">
+      <c r="J16" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="169" t="s">
+      <c r="A17" s="155" t="s">
         <v>183</v>
       </c>
-      <c r="B17" s="178">
+      <c r="B17" s="162">
         <v>3.9211523567242897E-2</v>
       </c>
-      <c r="C17" s="179">
+      <c r="C17" s="163">
         <v>6.4800724140040705E-2</v>
       </c>
-      <c r="D17" s="180">
+      <c r="D17" s="164">
         <v>9.0389924712838396E-2</v>
       </c>
-      <c r="E17" s="179">
+      <c r="E17" s="163">
         <v>0.14797197236920701</v>
       </c>
-      <c r="F17" s="181">
+      <c r="F17" s="165">
         <v>0.43792566323543602</v>
       </c>
-      <c r="G17" s="179">
+      <c r="G17" s="163">
         <v>8.98007241400407E-2</v>
       </c>
-      <c r="H17" s="182">
+      <c r="H17" s="166">
         <v>0.7</v>
       </c>
-      <c r="I17" s="183">
+      <c r="I17" s="167">
         <v>32720</v>
       </c>
-      <c r="J17" s="183">
+      <c r="J17" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" s="199" t="s">
+      <c r="A18" s="183" t="s">
         <v>148</v>
       </c>
-      <c r="B18" s="200">
+      <c r="B18" s="184">
         <v>1.6403181443203799E-2</v>
       </c>
-      <c r="C18" s="201">
+      <c r="C18" s="185">
         <v>4.4976836696510598E-2</v>
       </c>
-      <c r="D18" s="202">
+      <c r="D18" s="186">
         <v>7.3550491949817401E-2</v>
       </c>
-      <c r="E18" s="201">
+      <c r="E18" s="185">
         <v>0.139789727557039</v>
       </c>
-      <c r="F18" s="203">
+      <c r="F18" s="187">
         <v>0.32174636493341902</v>
       </c>
-      <c r="G18" s="201">
+      <c r="G18" s="185">
         <v>6.99768366965106E-2</v>
       </c>
-      <c r="H18" s="204">
+      <c r="H18" s="188">
         <v>0.7</v>
       </c>
-      <c r="I18" s="205">
+      <c r="I18" s="189">
         <v>36189</v>
       </c>
-      <c r="J18" s="205">
+      <c r="J18" s="189">
         <v>45777</v>
       </c>
     </row>
-    <row r="19" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="192" t="s">
+    <row r="19" spans="1:10" s="154" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="176" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="193"/>
-      <c r="C19" s="194"/>
-      <c r="D19" s="195"/>
-      <c r="E19" s="194"/>
-      <c r="F19" s="196"/>
-      <c r="G19" s="194"/>
-      <c r="H19" s="197"/>
-      <c r="I19" s="198"/>
-      <c r="J19" s="198"/>
+      <c r="B19" s="177"/>
+      <c r="C19" s="178"/>
+      <c r="D19" s="179"/>
+      <c r="E19" s="178"/>
+      <c r="F19" s="180"/>
+      <c r="G19" s="178"/>
+      <c r="H19" s="181"/>
+      <c r="I19" s="182"/>
+      <c r="J19" s="182"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" s="169" t="s">
+      <c r="A20" s="155" t="s">
         <v>184</v>
       </c>
-      <c r="B20" s="178">
+      <c r="B20" s="162">
         <v>7.6750631221554899E-3</v>
       </c>
-      <c r="C20" s="179">
+      <c r="C20" s="163">
         <v>1.9169505465816701E-2</v>
       </c>
-      <c r="D20" s="180">
+      <c r="D20" s="164">
         <v>3.0663947809477999E-2</v>
       </c>
-      <c r="E20" s="179">
+      <c r="E20" s="163">
         <v>6.1826317761391997E-2</v>
       </c>
-      <c r="F20" s="191">
+      <c r="F20" s="175">
         <v>0.31005413487178901</v>
       </c>
-      <c r="G20" s="179">
+      <c r="G20" s="163">
         <v>4.41695054658168E-2</v>
       </c>
-      <c r="H20" s="182">
+      <c r="H20" s="166">
         <v>1</v>
       </c>
-      <c r="I20" s="183">
+      <c r="I20" s="167">
         <v>34365</v>
       </c>
-      <c r="J20" s="183">
+      <c r="J20" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="169" t="s">
+      <c r="A21" s="155" t="s">
         <v>185</v>
       </c>
-      <c r="B21" s="178">
+      <c r="B21" s="162">
         <v>4.3657888915111303E-3</v>
       </c>
-      <c r="C21" s="179">
+      <c r="C21" s="163">
         <v>2.0771382280796301E-2</v>
       </c>
-      <c r="D21" s="180">
+      <c r="D21" s="164">
         <v>3.7176975670081602E-2</v>
       </c>
-      <c r="E21" s="179">
+      <c r="E21" s="163">
         <v>8.8242421826534606E-2</v>
       </c>
-      <c r="F21" s="181">
+      <c r="F21" s="165">
         <v>0.23538998421449001</v>
       </c>
-      <c r="G21" s="179">
+      <c r="G21" s="163">
         <v>4.5771382280796302E-2</v>
       </c>
-      <c r="H21" s="182">
+      <c r="H21" s="166">
         <v>1</v>
       </c>
-      <c r="I21" s="183">
+      <c r="I21" s="167">
         <v>34365</v>
       </c>
-      <c r="J21" s="183">
+      <c r="J21" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="199" t="s">
+      <c r="A22" s="183" t="s">
         <v>140</v>
       </c>
-      <c r="B22" s="200">
+      <c r="B22" s="184">
         <v>3.4812134452342201E-3</v>
       </c>
-      <c r="C22" s="201">
+      <c r="C22" s="185">
         <v>1.8658048030354601E-2</v>
       </c>
-      <c r="D22" s="202">
+      <c r="D22" s="186">
         <v>3.3834882615475001E-2</v>
       </c>
-      <c r="E22" s="201">
+      <c r="E22" s="185">
         <v>8.1633172764504602E-2</v>
       </c>
-      <c r="F22" s="203">
+      <c r="F22" s="187">
         <v>0.228559633277753</v>
       </c>
-      <c r="G22" s="201">
+      <c r="G22" s="185">
         <v>4.3658048030354599E-2</v>
       </c>
-      <c r="H22" s="204">
+      <c r="H22" s="188">
         <v>1</v>
       </c>
-      <c r="I22" s="205">
+      <c r="I22" s="189">
         <v>34365</v>
       </c>
-      <c r="J22" s="205">
+      <c r="J22" s="189">
         <v>45777</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="192" t="s">
+    <row r="23" spans="1:10" s="154" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="176" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="193"/>
-      <c r="C23" s="194"/>
-      <c r="D23" s="195"/>
-      <c r="E23" s="194"/>
-      <c r="F23" s="196"/>
-      <c r="G23" s="194"/>
-      <c r="H23" s="197"/>
-      <c r="I23" s="198"/>
-      <c r="J23" s="198"/>
+      <c r="B23" s="177"/>
+      <c r="C23" s="178"/>
+      <c r="D23" s="179"/>
+      <c r="E23" s="178"/>
+      <c r="F23" s="180"/>
+      <c r="G23" s="178"/>
+      <c r="H23" s="181"/>
+      <c r="I23" s="182"/>
+      <c r="J23" s="182"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="169" t="s">
+      <c r="A24" s="155" t="s">
         <v>145</v>
       </c>
-      <c r="B24" s="178">
+      <c r="B24" s="162">
         <v>2.6608812004023499E-2</v>
       </c>
-      <c r="C24" s="179">
+      <c r="C24" s="163">
         <v>5.0216749358222103E-2</v>
       </c>
-      <c r="D24" s="180">
+      <c r="D24" s="164">
         <v>7.3824686712420803E-2</v>
       </c>
-      <c r="E24" s="179">
+      <c r="E24" s="163">
         <v>0.14763853637333799</v>
       </c>
-      <c r="F24" s="181">
+      <c r="F24" s="165">
         <v>0.340133074952987</v>
       </c>
-      <c r="G24" s="179">
+      <c r="G24" s="163">
         <v>7.5216749358222104E-2</v>
       </c>
-      <c r="H24" s="182">
+      <c r="H24" s="166">
         <v>0</v>
       </c>
-      <c r="I24" s="183">
+      <c r="I24" s="167">
         <v>25598</v>
       </c>
-      <c r="J24" s="183">
+      <c r="J24" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="169" t="s">
+      <c r="A25" s="155" t="s">
         <v>186</v>
       </c>
-      <c r="B25" s="178">
+      <c r="B25" s="162">
         <v>1.78707608365977E-2</v>
       </c>
-      <c r="C25" s="179">
+      <c r="C25" s="163">
         <v>3.5944264317563202E-2</v>
       </c>
-      <c r="D25" s="180">
+      <c r="D25" s="164">
         <v>5.40177677985288E-2</v>
       </c>
-      <c r="E25" s="179">
+      <c r="E25" s="163">
         <v>9.7213778264937697E-2</v>
       </c>
-      <c r="F25" s="181">
+      <c r="F25" s="165">
         <v>0.369744546082799</v>
       </c>
-      <c r="G25" s="179">
+      <c r="G25" s="163">
         <v>6.0944264317563203E-2</v>
       </c>
-      <c r="H25" s="182">
+      <c r="H25" s="166">
         <v>0</v>
       </c>
-      <c r="I25" s="183">
+      <c r="I25" s="167">
         <v>34365</v>
       </c>
-      <c r="J25" s="183">
+      <c r="J25" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="199" t="s">
+      <c r="A26" s="183" t="s">
         <v>147</v>
       </c>
-      <c r="B26" s="200">
+      <c r="B26" s="184">
         <v>1.3852677823030299E-2</v>
       </c>
-      <c r="C26" s="201">
+      <c r="C26" s="185">
         <v>4.7598983442139302E-2</v>
       </c>
-      <c r="D26" s="202">
+      <c r="D26" s="186">
         <v>8.1345289061248299E-2</v>
       </c>
-      <c r="E26" s="201">
+      <c r="E26" s="185">
         <v>0.21081962919687999</v>
       </c>
-      <c r="F26" s="203">
+      <c r="F26" s="187">
         <v>0.225780605076804</v>
       </c>
-      <c r="G26" s="201">
+      <c r="G26" s="185">
         <v>7.2598983442139303E-2</v>
       </c>
-      <c r="H26" s="204">
+      <c r="H26" s="188">
         <v>0</v>
       </c>
-      <c r="I26" s="205">
+      <c r="I26" s="189">
         <v>30680</v>
       </c>
-      <c r="J26" s="205">
+      <c r="J26" s="189">
         <v>44925</v>
       </c>
     </row>
-    <row r="27" spans="1:10" s="168" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="192" t="s">
+    <row r="27" spans="1:10" s="154" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="176" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="193"/>
-      <c r="C27" s="194"/>
-      <c r="D27" s="195"/>
-      <c r="E27" s="194"/>
-      <c r="F27" s="196"/>
-      <c r="G27" s="194"/>
-      <c r="H27" s="197"/>
-      <c r="I27" s="198"/>
-      <c r="J27" s="198"/>
+      <c r="B27" s="177"/>
+      <c r="C27" s="178"/>
+      <c r="D27" s="179"/>
+      <c r="E27" s="178"/>
+      <c r="F27" s="180"/>
+      <c r="G27" s="178"/>
+      <c r="H27" s="181"/>
+      <c r="I27" s="182"/>
+      <c r="J27" s="182"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="169" t="s">
+      <c r="A28" s="155" t="s">
         <v>142</v>
       </c>
-      <c r="B28" s="178">
+      <c r="B28" s="162">
         <v>2.64039774019777E-2</v>
       </c>
-      <c r="C28" s="179">
+      <c r="C28" s="163">
         <v>4.3364015406650899E-2</v>
       </c>
-      <c r="D28" s="180">
+      <c r="D28" s="164">
         <v>6.0324053411324102E-2</v>
       </c>
-      <c r="E28" s="179">
+      <c r="E28" s="163">
         <v>0.106064123700363</v>
       </c>
-      <c r="F28" s="181">
+      <c r="F28" s="165">
         <v>0.40884715673658401</v>
       </c>
-      <c r="G28" s="179">
+      <c r="G28" s="163">
         <v>6.8364015406650894E-2</v>
       </c>
-      <c r="H28" s="182">
+      <c r="H28" s="166">
         <v>0</v>
       </c>
-      <c r="I28" s="183">
+      <c r="I28" s="167">
         <v>30589</v>
       </c>
-      <c r="J28" s="183">
+      <c r="J28" s="167">
         <v>45777</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" s="169" t="s">
+      <c r="A29" s="155" t="s">
         <v>187</v>
       </c>
-      <c r="B29" s="178">
+      <c r="B29" s="162">
         <v>3.9132178171297799E-2</v>
       </c>
-      <c r="C29" s="179">
+      <c r="C29" s="163">
         <v>6.2011235623535797E-2</v>
       </c>
-      <c r="D29" s="180">
+      <c r="D29" s="164">
         <v>8.4890293075773796E-2</v>
       </c>
-      <c r="E29" s="179">
+      <c r="E29" s="163">
         <v>0.143080291393996</v>
       </c>
-      <c r="F29" s="181">
+      <c r="F29" s="165">
         <v>0.43340165874262299</v>
       </c>
-      <c r="G29" s="179">
+      <c r="G29" s="163">
         <v>8.7011235623535799E-2</v>
       </c>
-      <c r="H29" s="182">
+      <c r="H29" s="166">
         <v>0</v>
       </c>
-      <c r="I29" s="183">
+      <c r="I29" s="167">
         <v>30650</v>
       </c>
-      <c r="J29" s="183">
+      <c r="J29" s="167">
         <v>44925</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" s="184" t="s">
+      <c r="A30" s="168" t="s">
         <v>144</v>
       </c>
-      <c r="B30" s="185">
+      <c r="B30" s="169">
         <v>1.3852677823030299E-2</v>
       </c>
-      <c r="C30" s="186">
+      <c r="C30" s="170">
         <v>4.7598983442139302E-2</v>
       </c>
-      <c r="D30" s="187">
+      <c r="D30" s="171">
         <v>8.1345289061248299E-2</v>
       </c>
-      <c r="E30" s="186">
+      <c r="E30" s="170">
         <v>0.21081962919687999</v>
       </c>
-      <c r="F30" s="188">
+      <c r="F30" s="172">
         <v>0.225780605076804</v>
       </c>
-      <c r="G30" s="186">
+      <c r="G30" s="170">
         <v>7.2598983442139303E-2</v>
       </c>
-      <c r="H30" s="189">
+      <c r="H30" s="173">
         <v>0</v>
       </c>
-      <c r="I30" s="190">
+      <c r="I30" s="174">
         <v>30680</v>
       </c>
-      <c r="J30" s="190">
+      <c r="J30" s="174">
         <v>44925</v>
       </c>
     </row>
@@ -7797,19 +7834,19 @@
   <sheetData>
     <row r="1" spans="1:13" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="166" t="s">
+      <c r="B1" s="205" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="166"/>
-      <c r="D1" s="166"/>
-      <c r="E1" s="166"/>
-      <c r="F1" s="166"/>
-      <c r="G1" s="166"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="205"/>
+      <c r="F1" s="205"/>
+      <c r="G1" s="205"/>
       <c r="H1" s="91"/>
-      <c r="I1" s="166" t="s">
+      <c r="I1" s="205" t="s">
         <v>155</v>
       </c>
-      <c r="J1" s="166"/>
+      <c r="J1" s="205"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>

</xml_diff>